<commit_message>
added control pictures unicode block
</commit_message>
<xml_diff>
--- a/PUA_allocation_chart.xlsx
+++ b/PUA_allocation_chart.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="139">
   <si>
     <t xml:space="preserve">PUA Allocation Chart U+Fxxxx</t>
   </si>
@@ -128,6 +128,18 @@
     <t xml:space="preserve">Codestyle ASCII Variants</t>
   </si>
   <si>
+    <t xml:space="preserve">Hangul Jamo Variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1E6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1E7</t>
+  </si>
+  <si>
     <t xml:space="preserve">Small ASCII Characters for Super/Subscript Composition Used Internally</t>
   </si>
   <si>
@@ -417,9 +429,6 @@
   </si>
   <si>
     <t xml:space="preserve">F02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">…</t>
   </si>
   <si>
     <t xml:space="preserve">FFD</t>
@@ -599,7 +608,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -641,10 +650,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -939,15 +944,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U149"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:U166"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15.4" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="6.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="3" style="3" width="5"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2985,7 +2990,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B69,1)</f>
         <v>F050</v>
@@ -3009,7 +3014,7 @@
       <c r="Q85" s="10"/>
       <c r="R85" s="10"/>
     </row>
-    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B70,1)</f>
         <v>F051</v>
@@ -3031,712 +3036,662 @@
       <c r="Q86" s="10"/>
       <c r="R86" s="10"/>
     </row>
-    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B87" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B71,1)</f>
         <v>F052</v>
       </c>
-      <c r="C87" s="11" t="s">
+      <c r="C87" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D87" s="11"/>
-      <c r="E87" s="11"/>
-      <c r="F87" s="11"/>
-      <c r="G87" s="11"/>
-      <c r="H87" s="11"/>
-      <c r="I87" s="11"/>
-      <c r="J87" s="11"/>
-      <c r="K87" s="11"/>
-      <c r="L87" s="11"/>
-      <c r="M87" s="11"/>
-      <c r="N87" s="11"/>
-      <c r="O87" s="11"/>
-      <c r="P87" s="11"/>
-      <c r="Q87" s="11"/>
-      <c r="R87" s="11"/>
-    </row>
-    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D87" s="10"/>
+      <c r="E87" s="10"/>
+      <c r="F87" s="10"/>
+      <c r="G87" s="10"/>
+      <c r="H87" s="10"/>
+      <c r="I87" s="10"/>
+      <c r="J87" s="10"/>
+      <c r="K87" s="10"/>
+      <c r="L87" s="10"/>
+      <c r="M87" s="10"/>
+      <c r="N87" s="10"/>
+      <c r="O87" s="10"/>
+      <c r="P87" s="10"/>
+      <c r="Q87" s="10"/>
+      <c r="R87" s="10"/>
+    </row>
+    <row r="88" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B88" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B72,1)</f>
         <v>F053</v>
       </c>
-      <c r="C88" s="11"/>
-      <c r="D88" s="11"/>
-      <c r="E88" s="11"/>
-      <c r="F88" s="11"/>
-      <c r="G88" s="11"/>
-      <c r="H88" s="11"/>
-      <c r="I88" s="11"/>
-      <c r="J88" s="11"/>
-      <c r="K88" s="11"/>
-      <c r="L88" s="11"/>
-      <c r="M88" s="11"/>
-      <c r="N88" s="11"/>
-      <c r="O88" s="11"/>
-      <c r="P88" s="11"/>
-      <c r="Q88" s="11"/>
-      <c r="R88" s="11"/>
-    </row>
-    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C88" s="10"/>
+      <c r="D88" s="10"/>
+      <c r="E88" s="10"/>
+      <c r="F88" s="10"/>
+      <c r="G88" s="10"/>
+      <c r="H88" s="10"/>
+      <c r="I88" s="10"/>
+      <c r="J88" s="10"/>
+      <c r="K88" s="10"/>
+      <c r="L88" s="10"/>
+      <c r="M88" s="10"/>
+      <c r="N88" s="10"/>
+      <c r="O88" s="10"/>
+      <c r="P88" s="10"/>
+      <c r="Q88" s="10"/>
+      <c r="R88" s="10"/>
+    </row>
+    <row r="89" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B89" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B73,1)</f>
         <v>F054</v>
       </c>
-      <c r="C89" s="11"/>
-      <c r="D89" s="11"/>
-      <c r="E89" s="11"/>
-      <c r="F89" s="11"/>
-      <c r="G89" s="11"/>
-      <c r="H89" s="11"/>
-      <c r="I89" s="11"/>
-      <c r="J89" s="11"/>
-      <c r="K89" s="11"/>
-      <c r="L89" s="11"/>
-      <c r="M89" s="11"/>
-      <c r="N89" s="11"/>
-      <c r="O89" s="11"/>
-      <c r="P89" s="11"/>
-      <c r="Q89" s="11"/>
-      <c r="R89" s="11"/>
-    </row>
-    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C89" s="10"/>
+      <c r="D89" s="10"/>
+      <c r="E89" s="10"/>
+      <c r="F89" s="10"/>
+      <c r="G89" s="10"/>
+      <c r="H89" s="10"/>
+      <c r="I89" s="10"/>
+      <c r="J89" s="10"/>
+      <c r="K89" s="10"/>
+      <c r="L89" s="10"/>
+      <c r="M89" s="10"/>
+      <c r="N89" s="10"/>
+      <c r="O89" s="10"/>
+      <c r="P89" s="10"/>
+      <c r="Q89" s="10"/>
+      <c r="R89" s="10"/>
+    </row>
+    <row r="90" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B90" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B74,1)</f>
         <v>F055</v>
       </c>
-      <c r="C90" s="11"/>
-      <c r="D90" s="11"/>
-      <c r="E90" s="11"/>
-      <c r="F90" s="11"/>
-      <c r="G90" s="11"/>
-      <c r="H90" s="11"/>
-      <c r="I90" s="11"/>
-      <c r="J90" s="11"/>
-      <c r="K90" s="11"/>
-      <c r="L90" s="11"/>
-      <c r="M90" s="11"/>
-      <c r="N90" s="11"/>
-      <c r="O90" s="11"/>
-      <c r="P90" s="11"/>
-      <c r="Q90" s="11"/>
-      <c r="R90" s="11"/>
-    </row>
-    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C90" s="10"/>
+      <c r="D90" s="10"/>
+      <c r="E90" s="10"/>
+      <c r="F90" s="10"/>
+      <c r="G90" s="10"/>
+      <c r="H90" s="10"/>
+      <c r="I90" s="10"/>
+      <c r="J90" s="10"/>
+      <c r="K90" s="10"/>
+      <c r="L90" s="10"/>
+      <c r="M90" s="10"/>
+      <c r="N90" s="10"/>
+      <c r="O90" s="10"/>
+      <c r="P90" s="10"/>
+      <c r="Q90" s="10"/>
+      <c r="R90" s="10"/>
+    </row>
+    <row r="91" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B91" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B75,1)</f>
         <v>F056</v>
       </c>
-      <c r="C91" s="11"/>
-      <c r="D91" s="11"/>
-      <c r="E91" s="11"/>
-      <c r="F91" s="11"/>
-      <c r="G91" s="11"/>
-      <c r="H91" s="11"/>
-      <c r="I91" s="11"/>
-      <c r="J91" s="11"/>
-      <c r="K91" s="11"/>
-      <c r="L91" s="11"/>
-      <c r="M91" s="11"/>
-      <c r="N91" s="11"/>
-      <c r="O91" s="11"/>
-      <c r="P91" s="11"/>
-      <c r="Q91" s="11"/>
-      <c r="R91" s="11"/>
-    </row>
-    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C91" s="10"/>
+      <c r="D91" s="10"/>
+      <c r="E91" s="10"/>
+      <c r="F91" s="10"/>
+      <c r="G91" s="10"/>
+      <c r="H91" s="10"/>
+      <c r="I91" s="10"/>
+      <c r="J91" s="10"/>
+      <c r="K91" s="10"/>
+      <c r="L91" s="10"/>
+      <c r="M91" s="10"/>
+      <c r="N91" s="10"/>
+      <c r="O91" s="10"/>
+      <c r="P91" s="10"/>
+      <c r="Q91" s="10"/>
+      <c r="R91" s="10"/>
+    </row>
+    <row r="92" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B92" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B76,1)</f>
         <v>F057</v>
       </c>
-      <c r="C92" s="11"/>
-      <c r="D92" s="11"/>
-      <c r="E92" s="11"/>
-      <c r="F92" s="11"/>
-      <c r="G92" s="11"/>
-      <c r="H92" s="11"/>
-      <c r="I92" s="11"/>
-      <c r="J92" s="11"/>
-      <c r="K92" s="11"/>
-      <c r="L92" s="11"/>
-      <c r="M92" s="11"/>
-      <c r="N92" s="11"/>
-      <c r="O92" s="11"/>
-      <c r="P92" s="11"/>
-      <c r="Q92" s="11"/>
-      <c r="R92" s="11"/>
+      <c r="C92" s="10"/>
+      <c r="D92" s="10"/>
+      <c r="E92" s="10"/>
+      <c r="F92" s="10"/>
+      <c r="G92" s="10"/>
+      <c r="H92" s="10"/>
+      <c r="I92" s="10"/>
+      <c r="J92" s="10"/>
+      <c r="K92" s="10"/>
+      <c r="L92" s="10"/>
+      <c r="M92" s="10"/>
+      <c r="N92" s="10"/>
+      <c r="O92" s="10"/>
+      <c r="P92" s="10"/>
+      <c r="Q92" s="10"/>
+      <c r="R92" s="10"/>
     </row>
     <row r="93" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B93" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B77,1)</f>
         <v>F058</v>
       </c>
-      <c r="C93" s="12"/>
-      <c r="D93" s="12"/>
-      <c r="E93" s="12"/>
-      <c r="F93" s="12"/>
-      <c r="G93" s="12"/>
-      <c r="H93" s="12"/>
-      <c r="I93" s="12"/>
-      <c r="J93" s="12"/>
-      <c r="K93" s="12"/>
-      <c r="L93" s="12"/>
-      <c r="M93" s="12"/>
-      <c r="N93" s="12"/>
-      <c r="O93" s="12"/>
-      <c r="P93" s="12"/>
-      <c r="Q93" s="12"/>
-      <c r="R93" s="12"/>
+      <c r="C93" s="11"/>
+      <c r="D93" s="11"/>
+      <c r="E93" s="11"/>
+      <c r="F93" s="11"/>
+      <c r="G93" s="11"/>
+      <c r="H93" s="11"/>
+      <c r="I93" s="11"/>
+      <c r="J93" s="11"/>
+      <c r="K93" s="11"/>
+      <c r="L93" s="11"/>
+      <c r="M93" s="11"/>
+      <c r="N93" s="11"/>
+      <c r="O93" s="11"/>
+      <c r="P93" s="11"/>
+      <c r="Q93" s="11"/>
+      <c r="R93" s="11"/>
     </row>
     <row r="94" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B94" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B78,1)</f>
         <v>F059</v>
       </c>
-      <c r="C94" s="12"/>
-      <c r="D94" s="12"/>
-      <c r="E94" s="12"/>
-      <c r="F94" s="12"/>
-      <c r="G94" s="12"/>
-      <c r="H94" s="12"/>
-      <c r="I94" s="12"/>
-      <c r="J94" s="12"/>
-      <c r="K94" s="12"/>
-      <c r="L94" s="12"/>
-      <c r="M94" s="12"/>
-      <c r="N94" s="12"/>
-      <c r="O94" s="12"/>
-      <c r="P94" s="12"/>
-      <c r="Q94" s="12"/>
-      <c r="R94" s="12"/>
+      <c r="C94" s="11"/>
+      <c r="D94" s="11"/>
+      <c r="E94" s="11"/>
+      <c r="F94" s="11"/>
+      <c r="G94" s="11"/>
+      <c r="H94" s="11"/>
+      <c r="I94" s="11"/>
+      <c r="J94" s="11"/>
+      <c r="K94" s="11"/>
+      <c r="L94" s="11"/>
+      <c r="M94" s="11"/>
+      <c r="N94" s="11"/>
+      <c r="O94" s="11"/>
+      <c r="P94" s="11"/>
+      <c r="Q94" s="11"/>
+      <c r="R94" s="11"/>
     </row>
     <row r="95" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B79,1)</f>
         <v>F05A</v>
       </c>
-      <c r="C95" s="12"/>
-      <c r="D95" s="12"/>
-      <c r="E95" s="12"/>
-      <c r="F95" s="12"/>
-      <c r="G95" s="12"/>
-      <c r="H95" s="12"/>
-      <c r="I95" s="12"/>
-      <c r="J95" s="12"/>
-      <c r="K95" s="12"/>
-      <c r="L95" s="12"/>
-      <c r="M95" s="12"/>
-      <c r="N95" s="12"/>
-      <c r="O95" s="12"/>
-      <c r="P95" s="12"/>
-      <c r="Q95" s="12"/>
-      <c r="R95" s="12"/>
+      <c r="C95" s="11"/>
+      <c r="D95" s="11"/>
+      <c r="E95" s="11"/>
+      <c r="F95" s="11"/>
+      <c r="G95" s="11"/>
+      <c r="H95" s="11"/>
+      <c r="I95" s="11"/>
+      <c r="J95" s="11"/>
+      <c r="K95" s="11"/>
+      <c r="L95" s="11"/>
+      <c r="M95" s="11"/>
+      <c r="N95" s="11"/>
+      <c r="O95" s="11"/>
+      <c r="P95" s="11"/>
+      <c r="Q95" s="11"/>
+      <c r="R95" s="11"/>
     </row>
     <row r="96" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B80,1)</f>
         <v>F05B</v>
       </c>
-      <c r="C96" s="12"/>
-      <c r="D96" s="12"/>
-      <c r="E96" s="12"/>
-      <c r="F96" s="12"/>
-      <c r="G96" s="12"/>
-      <c r="H96" s="12"/>
-      <c r="I96" s="12"/>
-      <c r="J96" s="12"/>
-      <c r="K96" s="12"/>
-      <c r="L96" s="12"/>
-      <c r="M96" s="12"/>
-      <c r="N96" s="12"/>
-      <c r="O96" s="12"/>
-      <c r="P96" s="12"/>
-      <c r="Q96" s="12"/>
-      <c r="R96" s="12"/>
+      <c r="C96" s="11"/>
+      <c r="D96" s="11"/>
+      <c r="E96" s="11"/>
+      <c r="F96" s="11"/>
+      <c r="G96" s="11"/>
+      <c r="H96" s="11"/>
+      <c r="I96" s="11"/>
+      <c r="J96" s="11"/>
+      <c r="K96" s="11"/>
+      <c r="L96" s="11"/>
+      <c r="M96" s="11"/>
+      <c r="N96" s="11"/>
+      <c r="O96" s="11"/>
+      <c r="P96" s="11"/>
+      <c r="Q96" s="11"/>
+      <c r="R96" s="11"/>
     </row>
     <row r="97" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B81,1)</f>
         <v>F05C</v>
       </c>
-      <c r="C97" s="12"/>
-      <c r="D97" s="12"/>
-      <c r="E97" s="12"/>
-      <c r="F97" s="12"/>
-      <c r="G97" s="12"/>
-      <c r="H97" s="12"/>
-      <c r="I97" s="12"/>
-      <c r="J97" s="12"/>
-      <c r="K97" s="12"/>
-      <c r="L97" s="12"/>
-      <c r="M97" s="12"/>
-      <c r="N97" s="12"/>
-      <c r="O97" s="12"/>
-      <c r="P97" s="12"/>
-      <c r="Q97" s="12"/>
-      <c r="R97" s="12"/>
+      <c r="C97" s="11"/>
+      <c r="D97" s="11"/>
+      <c r="E97" s="11"/>
+      <c r="F97" s="11"/>
+      <c r="G97" s="11"/>
+      <c r="H97" s="11"/>
+      <c r="I97" s="11"/>
+      <c r="J97" s="11"/>
+      <c r="K97" s="11"/>
+      <c r="L97" s="11"/>
+      <c r="M97" s="11"/>
+      <c r="N97" s="11"/>
+      <c r="O97" s="11"/>
+      <c r="P97" s="11"/>
+      <c r="Q97" s="11"/>
+      <c r="R97" s="11"/>
     </row>
     <row r="98" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B82,1)</f>
         <v>F05D</v>
       </c>
-      <c r="C98" s="12"/>
-      <c r="D98" s="12"/>
-      <c r="E98" s="12"/>
-      <c r="F98" s="12"/>
-      <c r="G98" s="12"/>
-      <c r="H98" s="12"/>
-      <c r="I98" s="12"/>
-      <c r="J98" s="12"/>
-      <c r="K98" s="12"/>
-      <c r="L98" s="12"/>
-      <c r="M98" s="12"/>
-      <c r="N98" s="12"/>
-      <c r="O98" s="12"/>
-      <c r="P98" s="12"/>
-      <c r="Q98" s="12"/>
-      <c r="R98" s="12"/>
+      <c r="C98" s="11"/>
+      <c r="D98" s="11"/>
+      <c r="E98" s="11"/>
+      <c r="F98" s="11"/>
+      <c r="G98" s="11"/>
+      <c r="H98" s="11"/>
+      <c r="I98" s="11"/>
+      <c r="J98" s="11"/>
+      <c r="K98" s="11"/>
+      <c r="L98" s="11"/>
+      <c r="M98" s="11"/>
+      <c r="N98" s="11"/>
+      <c r="O98" s="11"/>
+      <c r="P98" s="11"/>
+      <c r="Q98" s="11"/>
+      <c r="R98" s="11"/>
     </row>
     <row r="99" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B83,1)</f>
         <v>F05E</v>
       </c>
-      <c r="C99" s="12"/>
-      <c r="D99" s="12"/>
-      <c r="E99" s="12"/>
-      <c r="F99" s="12"/>
-      <c r="G99" s="12"/>
-      <c r="H99" s="12"/>
-      <c r="I99" s="12"/>
-      <c r="J99" s="12"/>
-      <c r="K99" s="12"/>
-      <c r="L99" s="12"/>
-      <c r="M99" s="12"/>
-      <c r="N99" s="12"/>
-      <c r="O99" s="12"/>
-      <c r="P99" s="12"/>
-      <c r="Q99" s="12"/>
-      <c r="R99" s="12"/>
+      <c r="C99" s="11"/>
+      <c r="D99" s="11"/>
+      <c r="E99" s="11"/>
+      <c r="F99" s="11"/>
+      <c r="G99" s="11"/>
+      <c r="H99" s="11"/>
+      <c r="I99" s="11"/>
+      <c r="J99" s="11"/>
+      <c r="K99" s="11"/>
+      <c r="L99" s="11"/>
+      <c r="M99" s="11"/>
+      <c r="N99" s="11"/>
+      <c r="O99" s="11"/>
+      <c r="P99" s="11"/>
+      <c r="Q99" s="11"/>
+      <c r="R99" s="11"/>
     </row>
     <row r="100" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="2" t="str">
         <f aca="false">"F05"&amp;RIGHT(B84,1)</f>
         <v>F05F</v>
       </c>
-      <c r="C100" s="12"/>
-      <c r="D100" s="12"/>
-      <c r="E100" s="12"/>
-      <c r="F100" s="12"/>
-      <c r="G100" s="12"/>
-      <c r="H100" s="12"/>
-      <c r="I100" s="12"/>
-      <c r="J100" s="12"/>
-      <c r="K100" s="12"/>
-      <c r="L100" s="12"/>
-      <c r="M100" s="12"/>
-      <c r="N100" s="12"/>
-      <c r="O100" s="12"/>
-      <c r="P100" s="12"/>
-      <c r="Q100" s="12"/>
-      <c r="R100" s="12"/>
+      <c r="C100" s="11"/>
+      <c r="D100" s="11"/>
+      <c r="E100" s="11"/>
+      <c r="F100" s="11"/>
+      <c r="G100" s="11"/>
+      <c r="H100" s="11"/>
+      <c r="I100" s="11"/>
+      <c r="J100" s="11"/>
+      <c r="K100" s="11"/>
+      <c r="L100" s="11"/>
+      <c r="M100" s="11"/>
+      <c r="N100" s="11"/>
+      <c r="O100" s="11"/>
+      <c r="P100" s="11"/>
+      <c r="Q100" s="11"/>
+      <c r="R100" s="11"/>
     </row>
     <row r="101" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C101" s="12"/>
-      <c r="D101" s="12"/>
-      <c r="E101" s="12"/>
-      <c r="F101" s="12"/>
-      <c r="G101" s="12"/>
-      <c r="H101" s="12"/>
-      <c r="I101" s="12"/>
-      <c r="J101" s="12"/>
-      <c r="K101" s="12"/>
-      <c r="L101" s="12"/>
-      <c r="M101" s="12"/>
-      <c r="N101" s="12"/>
-      <c r="O101" s="12"/>
-      <c r="P101" s="12"/>
-      <c r="Q101" s="12"/>
-      <c r="R101" s="12"/>
+      <c r="B101" s="2" t="str">
+        <f aca="false">"F06"&amp;RIGHT(B85,1)</f>
+        <v>F060</v>
+      </c>
+      <c r="C101" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D101" s="10"/>
+      <c r="E101" s="10"/>
+      <c r="F101" s="10"/>
+      <c r="G101" s="10"/>
+      <c r="H101" s="10"/>
+      <c r="I101" s="10"/>
+      <c r="J101" s="10"/>
+      <c r="K101" s="10"/>
+      <c r="L101" s="10"/>
+      <c r="M101" s="10"/>
+      <c r="N101" s="10"/>
+      <c r="O101" s="10"/>
+      <c r="P101" s="10"/>
+      <c r="Q101" s="10"/>
+      <c r="R101" s="10"/>
+    </row>
+    <row r="102" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B102" s="2" t="str">
+        <f aca="false">"F06"&amp;RIGHT(B86,1)</f>
+        <v>F061</v>
+      </c>
+      <c r="C102" s="10"/>
+      <c r="D102" s="10"/>
+      <c r="E102" s="10"/>
+      <c r="F102" s="10"/>
+      <c r="G102" s="10"/>
+      <c r="H102" s="10"/>
+      <c r="I102" s="10"/>
+      <c r="J102" s="10"/>
+      <c r="K102" s="10"/>
+      <c r="L102" s="10"/>
+      <c r="M102" s="10"/>
+      <c r="N102" s="10"/>
+      <c r="O102" s="10"/>
+      <c r="P102" s="10"/>
+      <c r="Q102" s="10"/>
+      <c r="R102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B103" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C103" s="5"/>
-      <c r="D103" s="5"/>
-      <c r="E103" s="5"/>
-      <c r="F103" s="5"/>
-      <c r="G103" s="5"/>
-      <c r="H103" s="5"/>
-      <c r="I103" s="5"/>
-      <c r="J103" s="5"/>
-      <c r="K103" s="5"/>
-      <c r="L103" s="5"/>
-      <c r="M103" s="5"/>
-      <c r="N103" s="5"/>
-      <c r="O103" s="5"/>
-      <c r="P103" s="5"/>
-      <c r="Q103" s="5"/>
-      <c r="R103" s="5"/>
-      <c r="S103" s="1" t="s">
+      <c r="B103" s="2" t="s">
         <v>36</v>
       </c>
+      <c r="C103" s="10"/>
+      <c r="D103" s="10"/>
+      <c r="E103" s="10"/>
+      <c r="F103" s="10"/>
+      <c r="G103" s="10"/>
+      <c r="H103" s="10"/>
+      <c r="I103" s="10"/>
+      <c r="J103" s="10"/>
+      <c r="K103" s="10"/>
+      <c r="L103" s="10"/>
+      <c r="M103" s="10"/>
+      <c r="N103" s="10"/>
+      <c r="O103" s="10"/>
+      <c r="P103" s="10"/>
+      <c r="Q103" s="10"/>
+      <c r="R103" s="10"/>
     </row>
     <row r="104" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B104" s="6"/>
-      <c r="C104" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D104" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E104" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F104" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G104" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H104" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I104" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J104" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K104" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L104" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="M104" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="N104" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O104" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P104" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q104" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="R104" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="B104" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C104" s="10"/>
+      <c r="D104" s="10"/>
+      <c r="E104" s="10"/>
+      <c r="F104" s="10"/>
+      <c r="G104" s="10"/>
+      <c r="H104" s="10"/>
+      <c r="I104" s="10"/>
+      <c r="J104" s="10"/>
+      <c r="K104" s="10"/>
+      <c r="L104" s="10"/>
+      <c r="M104" s="10"/>
+      <c r="N104" s="10"/>
+      <c r="O104" s="10"/>
+      <c r="P104" s="10"/>
+      <c r="Q104" s="10"/>
+      <c r="R104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B105" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C105" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D105" s="13"/>
-      <c r="E105" s="13"/>
-      <c r="F105" s="13"/>
-      <c r="G105" s="13"/>
-      <c r="H105" s="13"/>
-      <c r="I105" s="13"/>
-      <c r="J105" s="13"/>
-      <c r="K105" s="13"/>
-      <c r="L105" s="13"/>
-      <c r="M105" s="13"/>
-      <c r="N105" s="13"/>
-      <c r="O105" s="13"/>
-      <c r="P105" s="13"/>
-      <c r="Q105" s="13"/>
-      <c r="R105" s="13"/>
-      <c r="S105" s="14" t="s">
-        <v>39</v>
-      </c>
+      <c r="C105" s="10"/>
+      <c r="D105" s="10"/>
+      <c r="E105" s="10"/>
+      <c r="F105" s="10"/>
+      <c r="G105" s="10"/>
+      <c r="H105" s="10"/>
+      <c r="I105" s="10"/>
+      <c r="J105" s="10"/>
+      <c r="K105" s="10"/>
+      <c r="L105" s="10"/>
+      <c r="M105" s="10"/>
+      <c r="N105" s="10"/>
+      <c r="O105" s="10"/>
+      <c r="P105" s="10"/>
+      <c r="Q105" s="10"/>
+      <c r="R105" s="10"/>
     </row>
     <row r="106" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B106" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C106" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="D106" s="13"/>
-      <c r="E106" s="13"/>
-      <c r="F106" s="13"/>
-      <c r="G106" s="13"/>
-      <c r="H106" s="13"/>
-      <c r="I106" s="13"/>
-      <c r="J106" s="13"/>
-      <c r="K106" s="13"/>
-      <c r="L106" s="13"/>
-      <c r="M106" s="13"/>
-      <c r="N106" s="13"/>
-      <c r="O106" s="13"/>
-      <c r="P106" s="13"/>
-      <c r="Q106" s="13"/>
-      <c r="R106" s="13"/>
+      <c r="C106" s="11"/>
+      <c r="D106" s="11"/>
+      <c r="E106" s="11"/>
+      <c r="F106" s="11"/>
+      <c r="G106" s="11"/>
+      <c r="H106" s="11"/>
+      <c r="I106" s="11"/>
+      <c r="J106" s="11"/>
+      <c r="K106" s="11"/>
+      <c r="L106" s="11"/>
+      <c r="M106" s="11"/>
+      <c r="N106" s="11"/>
+      <c r="O106" s="11"/>
+      <c r="P106" s="11"/>
+      <c r="Q106" s="11"/>
+      <c r="R106" s="11"/>
     </row>
     <row r="107" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B107" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C107" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="D107" s="13"/>
-      <c r="E107" s="13"/>
-      <c r="F107" s="13"/>
-      <c r="G107" s="13"/>
-      <c r="H107" s="13"/>
-      <c r="I107" s="13"/>
-      <c r="J107" s="13"/>
-      <c r="K107" s="13"/>
-      <c r="L107" s="13"/>
-      <c r="M107" s="13"/>
-      <c r="N107" s="13"/>
-      <c r="O107" s="13"/>
-      <c r="P107" s="13"/>
-      <c r="Q107" s="13"/>
-      <c r="R107" s="13"/>
+      <c r="C107" s="11"/>
+      <c r="D107" s="11"/>
+      <c r="E107" s="11"/>
+      <c r="F107" s="11"/>
+      <c r="G107" s="11"/>
+      <c r="H107" s="11"/>
+      <c r="I107" s="11"/>
+      <c r="J107" s="11"/>
+      <c r="K107" s="11"/>
+      <c r="L107" s="11"/>
+      <c r="M107" s="11"/>
+      <c r="N107" s="11"/>
+      <c r="O107" s="11"/>
+      <c r="P107" s="11"/>
+      <c r="Q107" s="11"/>
+      <c r="R107" s="11"/>
     </row>
     <row r="108" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B108" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C108" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D108" s="13"/>
-      <c r="E108" s="13"/>
-      <c r="F108" s="13"/>
-      <c r="G108" s="13"/>
-      <c r="H108" s="13"/>
-      <c r="I108" s="13"/>
-      <c r="J108" s="13"/>
-      <c r="K108" s="13"/>
-      <c r="L108" s="13"/>
-      <c r="M108" s="13"/>
-      <c r="N108" s="13"/>
-      <c r="O108" s="13"/>
-      <c r="P108" s="13"/>
-      <c r="Q108" s="13"/>
-      <c r="R108" s="13"/>
+      <c r="C108" s="11"/>
+      <c r="D108" s="11"/>
+      <c r="E108" s="11"/>
+      <c r="F108" s="11"/>
+      <c r="G108" s="11"/>
+      <c r="H108" s="11"/>
+      <c r="I108" s="11"/>
+      <c r="J108" s="11"/>
+      <c r="K108" s="11"/>
+      <c r="L108" s="11"/>
+      <c r="M108" s="11"/>
+      <c r="N108" s="11"/>
+      <c r="O108" s="11"/>
+      <c r="P108" s="11"/>
+      <c r="Q108" s="11"/>
+      <c r="R108" s="11"/>
     </row>
     <row r="109" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B109" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C109" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="D109" s="13"/>
-      <c r="E109" s="13"/>
-      <c r="F109" s="13"/>
-      <c r="G109" s="13"/>
-      <c r="H109" s="13"/>
-      <c r="I109" s="13"/>
-      <c r="J109" s="13"/>
-      <c r="K109" s="13"/>
-      <c r="L109" s="13"/>
-      <c r="M109" s="13"/>
-      <c r="N109" s="13"/>
-      <c r="O109" s="13"/>
-      <c r="P109" s="13"/>
-      <c r="Q109" s="13"/>
-      <c r="R109" s="13"/>
+      <c r="C109" s="11"/>
+      <c r="D109" s="11"/>
+      <c r="E109" s="11"/>
+      <c r="F109" s="11"/>
+      <c r="G109" s="11"/>
+      <c r="H109" s="11"/>
+      <c r="I109" s="11"/>
+      <c r="J109" s="11"/>
+      <c r="K109" s="11"/>
+      <c r="L109" s="11"/>
+      <c r="M109" s="11"/>
+      <c r="N109" s="11"/>
+      <c r="O109" s="11"/>
+      <c r="P109" s="11"/>
+      <c r="Q109" s="11"/>
+      <c r="R109" s="11"/>
     </row>
     <row r="110" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B110" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C110" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="D110" s="13"/>
-      <c r="E110" s="13"/>
-      <c r="F110" s="13"/>
-      <c r="G110" s="13"/>
-      <c r="H110" s="13"/>
-      <c r="I110" s="13"/>
-      <c r="J110" s="13"/>
-      <c r="K110" s="13"/>
-      <c r="L110" s="13"/>
-      <c r="M110" s="13"/>
-      <c r="N110" s="13"/>
-      <c r="O110" s="13"/>
-      <c r="P110" s="13"/>
-      <c r="Q110" s="13"/>
-      <c r="R110" s="13"/>
+      <c r="C110" s="11"/>
+      <c r="D110" s="11"/>
+      <c r="E110" s="11"/>
+      <c r="F110" s="11"/>
+      <c r="G110" s="11"/>
+      <c r="H110" s="11"/>
+      <c r="I110" s="11"/>
+      <c r="J110" s="11"/>
+      <c r="K110" s="11"/>
+      <c r="L110" s="11"/>
+      <c r="M110" s="11"/>
+      <c r="N110" s="11"/>
+      <c r="O110" s="11"/>
+      <c r="P110" s="11"/>
+      <c r="Q110" s="11"/>
+      <c r="R110" s="11"/>
+    </row>
+    <row r="111" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C111" s="11"/>
+      <c r="D111" s="11"/>
+      <c r="E111" s="11"/>
+      <c r="F111" s="11"/>
+      <c r="G111" s="11"/>
+      <c r="H111" s="11"/>
+      <c r="I111" s="11"/>
+      <c r="J111" s="11"/>
+      <c r="K111" s="11"/>
+      <c r="L111" s="11"/>
+      <c r="M111" s="11"/>
+      <c r="N111" s="11"/>
+      <c r="O111" s="11"/>
+      <c r="P111" s="11"/>
+      <c r="Q111" s="11"/>
+      <c r="R111" s="11"/>
     </row>
     <row r="112" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B112" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C112" s="5"/>
-      <c r="D112" s="5"/>
-      <c r="E112" s="5"/>
-      <c r="F112" s="5"/>
-      <c r="G112" s="5"/>
-      <c r="H112" s="5"/>
-      <c r="I112" s="5"/>
-      <c r="J112" s="5"/>
-      <c r="K112" s="5"/>
-      <c r="L112" s="5"/>
-      <c r="M112" s="5"/>
-      <c r="N112" s="5"/>
-      <c r="O112" s="5"/>
-      <c r="P112" s="5"/>
-      <c r="Q112" s="5"/>
-      <c r="R112" s="5"/>
+      <c r="C112" s="11"/>
+      <c r="D112" s="11"/>
+      <c r="E112" s="11"/>
+      <c r="F112" s="11"/>
+      <c r="G112" s="11"/>
+      <c r="H112" s="11"/>
+      <c r="I112" s="11"/>
+      <c r="J112" s="11"/>
+      <c r="K112" s="11"/>
+      <c r="L112" s="11"/>
+      <c r="M112" s="11"/>
+      <c r="N112" s="11"/>
+      <c r="O112" s="11"/>
+      <c r="P112" s="11"/>
+      <c r="Q112" s="11"/>
+      <c r="R112" s="11"/>
     </row>
     <row r="113" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B113" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C113" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D113" s="13"/>
-      <c r="E113" s="13"/>
-      <c r="F113" s="13"/>
-      <c r="G113" s="13"/>
-      <c r="H113" s="13"/>
-      <c r="I113" s="13"/>
-      <c r="J113" s="13"/>
-      <c r="K113" s="13"/>
-      <c r="L113" s="13"/>
-      <c r="M113" s="13"/>
-      <c r="N113" s="13"/>
-      <c r="O113" s="13"/>
-      <c r="P113" s="13"/>
-      <c r="Q113" s="13"/>
-      <c r="R113" s="13"/>
+      <c r="C113" s="11"/>
+      <c r="D113" s="11"/>
+      <c r="E113" s="11"/>
+      <c r="F113" s="11"/>
+      <c r="G113" s="11"/>
+      <c r="H113" s="11"/>
+      <c r="I113" s="11"/>
+      <c r="J113" s="11"/>
+      <c r="K113" s="11"/>
+      <c r="L113" s="11"/>
+      <c r="M113" s="11"/>
+      <c r="N113" s="11"/>
+      <c r="O113" s="11"/>
+      <c r="P113" s="11"/>
+      <c r="Q113" s="11"/>
+      <c r="R113" s="11"/>
     </row>
     <row r="114" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B114" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C114" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="D114" s="13"/>
-      <c r="E114" s="13"/>
-      <c r="F114" s="13"/>
-      <c r="G114" s="13"/>
-      <c r="H114" s="13"/>
-      <c r="I114" s="13"/>
-      <c r="J114" s="13"/>
-      <c r="K114" s="13"/>
-      <c r="L114" s="13"/>
-      <c r="M114" s="13"/>
-      <c r="N114" s="13"/>
-      <c r="O114" s="13"/>
-      <c r="P114" s="13"/>
-      <c r="Q114" s="13"/>
-      <c r="R114" s="13"/>
+      <c r="C114" s="11"/>
+      <c r="D114" s="11"/>
+      <c r="E114" s="11"/>
+      <c r="F114" s="11"/>
+      <c r="G114" s="11"/>
+      <c r="H114" s="11"/>
+      <c r="I114" s="11"/>
+      <c r="J114" s="11"/>
+      <c r="K114" s="11"/>
+      <c r="L114" s="11"/>
+      <c r="M114" s="11"/>
+      <c r="N114" s="11"/>
+      <c r="O114" s="11"/>
+      <c r="P114" s="11"/>
+      <c r="Q114" s="11"/>
+      <c r="R114" s="11"/>
     </row>
     <row r="115" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B115" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C115" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="D115" s="13"/>
-      <c r="E115" s="13"/>
-      <c r="F115" s="13"/>
-      <c r="G115" s="13"/>
-      <c r="H115" s="13"/>
-      <c r="I115" s="13"/>
-      <c r="J115" s="13"/>
-      <c r="K115" s="13"/>
-      <c r="L115" s="13"/>
-      <c r="M115" s="13"/>
-      <c r="N115" s="13"/>
-      <c r="O115" s="13"/>
-      <c r="P115" s="13"/>
-      <c r="Q115" s="13"/>
-      <c r="R115" s="13"/>
+      <c r="C115" s="11"/>
+      <c r="D115" s="11"/>
+      <c r="E115" s="11"/>
+      <c r="F115" s="11"/>
+      <c r="G115" s="11"/>
+      <c r="H115" s="11"/>
+      <c r="I115" s="11"/>
+      <c r="J115" s="11"/>
+      <c r="K115" s="11"/>
+      <c r="L115" s="11"/>
+      <c r="M115" s="11"/>
+      <c r="N115" s="11"/>
+      <c r="O115" s="11"/>
+      <c r="P115" s="11"/>
+      <c r="Q115" s="11"/>
+      <c r="R115" s="11"/>
     </row>
     <row r="116" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B116" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C116" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D116" s="13"/>
-      <c r="E116" s="13"/>
-      <c r="F116" s="13"/>
-      <c r="G116" s="13"/>
-      <c r="H116" s="13"/>
-      <c r="I116" s="13"/>
-      <c r="J116" s="13"/>
-      <c r="K116" s="13"/>
-      <c r="L116" s="13"/>
-      <c r="M116" s="13"/>
-      <c r="N116" s="13"/>
-      <c r="O116" s="13"/>
-      <c r="P116" s="13"/>
-      <c r="Q116" s="13"/>
-      <c r="R116" s="13"/>
+      <c r="C116" s="11"/>
+      <c r="D116" s="11"/>
+      <c r="E116" s="11"/>
+      <c r="F116" s="11"/>
+      <c r="G116" s="11"/>
+      <c r="H116" s="11"/>
+      <c r="I116" s="11"/>
+      <c r="J116" s="11"/>
+      <c r="K116" s="11"/>
+      <c r="L116" s="11"/>
+      <c r="M116" s="11"/>
+      <c r="N116" s="11"/>
+      <c r="O116" s="11"/>
+      <c r="P116" s="11"/>
+      <c r="Q116" s="11"/>
+      <c r="R116" s="11"/>
     </row>
     <row r="117" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B117" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C117" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="D117" s="13"/>
-      <c r="E117" s="13"/>
-      <c r="F117" s="13"/>
-      <c r="G117" s="13"/>
-      <c r="H117" s="13"/>
-      <c r="I117" s="13"/>
-      <c r="J117" s="13"/>
-      <c r="K117" s="13"/>
-      <c r="L117" s="13"/>
-      <c r="M117" s="13"/>
-      <c r="N117" s="13"/>
-      <c r="O117" s="13"/>
-      <c r="P117" s="13"/>
-      <c r="Q117" s="13"/>
-      <c r="R117" s="13"/>
+      <c r="C117" s="11"/>
+      <c r="D117" s="11"/>
+      <c r="E117" s="11"/>
+      <c r="F117" s="11"/>
+      <c r="G117" s="11"/>
+      <c r="H117" s="11"/>
+      <c r="I117" s="11"/>
+      <c r="J117" s="11"/>
+      <c r="K117" s="11"/>
+      <c r="L117" s="11"/>
+      <c r="M117" s="11"/>
+      <c r="N117" s="11"/>
+      <c r="O117" s="11"/>
+      <c r="P117" s="11"/>
+      <c r="Q117" s="11"/>
+      <c r="R117" s="11"/>
     </row>
     <row r="118" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B118" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C118" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="D118" s="13"/>
-      <c r="E118" s="13"/>
-      <c r="F118" s="13"/>
-      <c r="G118" s="13"/>
-      <c r="H118" s="13"/>
-      <c r="I118" s="13"/>
-      <c r="J118" s="13"/>
-      <c r="K118" s="13"/>
-      <c r="L118" s="13"/>
-      <c r="M118" s="13"/>
-      <c r="N118" s="13"/>
-      <c r="O118" s="13"/>
-      <c r="P118" s="13"/>
-      <c r="Q118" s="13"/>
-      <c r="R118" s="13"/>
+      <c r="C118" s="11"/>
+      <c r="D118" s="11"/>
+      <c r="E118" s="11"/>
+      <c r="F118" s="11"/>
+      <c r="G118" s="11"/>
+      <c r="H118" s="11"/>
+      <c r="I118" s="11"/>
+      <c r="J118" s="11"/>
+      <c r="K118" s="11"/>
+      <c r="L118" s="11"/>
+      <c r="M118" s="11"/>
+      <c r="N118" s="11"/>
+      <c r="O118" s="11"/>
+      <c r="P118" s="11"/>
+      <c r="Q118" s="11"/>
+      <c r="R118" s="11"/>
     </row>
     <row r="120" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B120" s="5" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="C120" s="5"/>
       <c r="D120" s="5"/>
@@ -3754,6 +3709,9 @@
       <c r="P120" s="5"/>
       <c r="Q120" s="5"/>
       <c r="R120" s="5"/>
+      <c r="S120" s="1" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B121" s="6"/>
@@ -3808,798 +3766,1167 @@
     </row>
     <row r="122" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B122" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C122" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D122" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="S122" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="T122" s="1" t="s">
-        <v>68</v>
+        <v>41</v>
+      </c>
+      <c r="C122" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D122" s="12"/>
+      <c r="E122" s="12"/>
+      <c r="F122" s="12"/>
+      <c r="G122" s="12"/>
+      <c r="H122" s="12"/>
+      <c r="I122" s="12"/>
+      <c r="J122" s="12"/>
+      <c r="K122" s="12"/>
+      <c r="L122" s="12"/>
+      <c r="M122" s="12"/>
+      <c r="N122" s="12"/>
+      <c r="O122" s="12"/>
+      <c r="P122" s="12"/>
+      <c r="Q122" s="12"/>
+      <c r="R122" s="12"/>
+      <c r="S122" s="13" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B123" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C123" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="S123" s="1" t="s">
-        <v>71</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="C123" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D123" s="12"/>
+      <c r="E123" s="12"/>
+      <c r="F123" s="12"/>
+      <c r="G123" s="12"/>
+      <c r="H123" s="12"/>
+      <c r="I123" s="12"/>
+      <c r="J123" s="12"/>
+      <c r="K123" s="12"/>
+      <c r="L123" s="12"/>
+      <c r="M123" s="12"/>
+      <c r="N123" s="12"/>
+      <c r="O123" s="12"/>
+      <c r="P123" s="12"/>
+      <c r="Q123" s="12"/>
+      <c r="R123" s="12"/>
     </row>
     <row r="124" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B124" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C124" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="D124" s="10"/>
-      <c r="E124" s="10"/>
-      <c r="F124" s="10"/>
-      <c r="G124" s="10"/>
-      <c r="H124" s="10"/>
-      <c r="I124" s="10"/>
-      <c r="J124" s="10"/>
-      <c r="K124" s="10"/>
-      <c r="L124" s="10"/>
-      <c r="M124" s="10"/>
-      <c r="N124" s="10"/>
-      <c r="O124" s="10"/>
-      <c r="P124" s="10"/>
-      <c r="Q124" s="10"/>
-      <c r="R124" s="10"/>
+        <v>46</v>
+      </c>
+      <c r="C124" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D124" s="12"/>
+      <c r="E124" s="12"/>
+      <c r="F124" s="12"/>
+      <c r="G124" s="12"/>
+      <c r="H124" s="12"/>
+      <c r="I124" s="12"/>
+      <c r="J124" s="12"/>
+      <c r="K124" s="12"/>
+      <c r="L124" s="12"/>
+      <c r="M124" s="12"/>
+      <c r="N124" s="12"/>
+      <c r="O124" s="12"/>
+      <c r="P124" s="12"/>
+      <c r="Q124" s="12"/>
+      <c r="R124" s="12"/>
     </row>
     <row r="125" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C125" s="10"/>
-      <c r="D125" s="10"/>
-      <c r="E125" s="10"/>
-      <c r="F125" s="10"/>
-      <c r="G125" s="10"/>
-      <c r="H125" s="10"/>
-      <c r="I125" s="10"/>
-      <c r="J125" s="10"/>
-      <c r="K125" s="10"/>
-      <c r="L125" s="10"/>
-      <c r="M125" s="10"/>
-      <c r="N125" s="10"/>
-      <c r="O125" s="10"/>
-      <c r="P125" s="10"/>
-      <c r="Q125" s="10"/>
-      <c r="R125" s="10"/>
-    </row>
-    <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B127" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C127" s="5"/>
-      <c r="D127" s="5"/>
-      <c r="E127" s="5"/>
-      <c r="F127" s="5"/>
-      <c r="G127" s="5"/>
-      <c r="H127" s="5"/>
-      <c r="I127" s="5"/>
-      <c r="J127" s="5"/>
-      <c r="K127" s="5"/>
-      <c r="L127" s="5"/>
-      <c r="M127" s="5"/>
-      <c r="N127" s="5"/>
-      <c r="O127" s="5"/>
-      <c r="P127" s="5"/>
-      <c r="Q127" s="5"/>
-      <c r="R127" s="5"/>
-      <c r="S127" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B128" s="6"/>
-      <c r="C128" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D128" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E128" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F128" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G128" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H128" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I128" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J128" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K128" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L128" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="M128" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="N128" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O128" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P128" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q128" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="R128" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B129" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C129" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D129" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E129" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F129" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G129" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H129" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="I129" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="J129" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="K129" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L129" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="M129" s="15"/>
-      <c r="N129" s="15"/>
-      <c r="O129" s="15"/>
-      <c r="P129" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q129" s="15"/>
-      <c r="R129" s="15"/>
-    </row>
-    <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>48</v>
+      </c>
+      <c r="C125" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D125" s="12"/>
+      <c r="E125" s="12"/>
+      <c r="F125" s="12"/>
+      <c r="G125" s="12"/>
+      <c r="H125" s="12"/>
+      <c r="I125" s="12"/>
+      <c r="J125" s="12"/>
+      <c r="K125" s="12"/>
+      <c r="L125" s="12"/>
+      <c r="M125" s="12"/>
+      <c r="N125" s="12"/>
+      <c r="O125" s="12"/>
+      <c r="P125" s="12"/>
+      <c r="Q125" s="12"/>
+      <c r="R125" s="12"/>
+    </row>
+    <row r="126" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B126" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C126" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D126" s="12"/>
+      <c r="E126" s="12"/>
+      <c r="F126" s="12"/>
+      <c r="G126" s="12"/>
+      <c r="H126" s="12"/>
+      <c r="I126" s="12"/>
+      <c r="J126" s="12"/>
+      <c r="K126" s="12"/>
+      <c r="L126" s="12"/>
+      <c r="M126" s="12"/>
+      <c r="N126" s="12"/>
+      <c r="O126" s="12"/>
+      <c r="P126" s="12"/>
+      <c r="Q126" s="12"/>
+      <c r="R126" s="12"/>
+    </row>
+    <row r="127" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B127" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C127" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D127" s="12"/>
+      <c r="E127" s="12"/>
+      <c r="F127" s="12"/>
+      <c r="G127" s="12"/>
+      <c r="H127" s="12"/>
+      <c r="I127" s="12"/>
+      <c r="J127" s="12"/>
+      <c r="K127" s="12"/>
+      <c r="L127" s="12"/>
+      <c r="M127" s="12"/>
+      <c r="N127" s="12"/>
+      <c r="O127" s="12"/>
+      <c r="P127" s="12"/>
+      <c r="Q127" s="12"/>
+      <c r="R127" s="12"/>
+    </row>
+    <row r="129" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B129" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C129" s="5"/>
+      <c r="D129" s="5"/>
+      <c r="E129" s="5"/>
+      <c r="F129" s="5"/>
+      <c r="G129" s="5"/>
+      <c r="H129" s="5"/>
+      <c r="I129" s="5"/>
+      <c r="J129" s="5"/>
+      <c r="K129" s="5"/>
+      <c r="L129" s="5"/>
+      <c r="M129" s="5"/>
+      <c r="N129" s="5"/>
+      <c r="O129" s="5"/>
+      <c r="P129" s="5"/>
+      <c r="Q129" s="5"/>
+      <c r="R129" s="5"/>
+    </row>
+    <row r="130" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C130" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D130" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E130" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F130" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G130" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H130" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I130" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J130" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="K130" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="L130" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="M130" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="N130" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="O130" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="P130" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q130" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="R130" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>55</v>
+      </c>
+      <c r="C130" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D130" s="12"/>
+      <c r="E130" s="12"/>
+      <c r="F130" s="12"/>
+      <c r="G130" s="12"/>
+      <c r="H130" s="12"/>
+      <c r="I130" s="12"/>
+      <c r="J130" s="12"/>
+      <c r="K130" s="12"/>
+      <c r="L130" s="12"/>
+      <c r="M130" s="12"/>
+      <c r="N130" s="12"/>
+      <c r="O130" s="12"/>
+      <c r="P130" s="12"/>
+      <c r="Q130" s="12"/>
+      <c r="R130" s="12"/>
+    </row>
+    <row r="131" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B131" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C131" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="D131" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E131" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="F131" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="G131" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="H131" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="I131" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="J131" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="K131" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="L131" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="M131" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="N131" s="15"/>
-      <c r="O131" s="15"/>
-      <c r="P131" s="15"/>
-      <c r="Q131" s="15"/>
-      <c r="R131" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>57</v>
+      </c>
+      <c r="C131" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D131" s="12"/>
+      <c r="E131" s="12"/>
+      <c r="F131" s="12"/>
+      <c r="G131" s="12"/>
+      <c r="H131" s="12"/>
+      <c r="I131" s="12"/>
+      <c r="J131" s="12"/>
+      <c r="K131" s="12"/>
+      <c r="L131" s="12"/>
+      <c r="M131" s="12"/>
+      <c r="N131" s="12"/>
+      <c r="O131" s="12"/>
+      <c r="P131" s="12"/>
+      <c r="Q131" s="12"/>
+      <c r="R131" s="12"/>
+    </row>
+    <row r="132" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B132" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C132" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D132" s="12"/>
+      <c r="E132" s="12"/>
+      <c r="F132" s="12"/>
+      <c r="G132" s="12"/>
+      <c r="H132" s="12"/>
+      <c r="I132" s="12"/>
+      <c r="J132" s="12"/>
+      <c r="K132" s="12"/>
+      <c r="L132" s="12"/>
+      <c r="M132" s="12"/>
+      <c r="N132" s="12"/>
+      <c r="O132" s="12"/>
+      <c r="P132" s="12"/>
+      <c r="Q132" s="12"/>
+      <c r="R132" s="12"/>
+    </row>
     <row r="133" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B133" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C133" s="5"/>
-      <c r="D133" s="5"/>
-      <c r="E133" s="5"/>
-      <c r="F133" s="5"/>
-      <c r="G133" s="5"/>
-      <c r="H133" s="5"/>
-      <c r="I133" s="5"/>
-      <c r="J133" s="5"/>
-      <c r="K133" s="5"/>
-      <c r="L133" s="5"/>
-      <c r="M133" s="5"/>
-      <c r="N133" s="5"/>
-      <c r="O133" s="5"/>
-      <c r="P133" s="5"/>
-      <c r="Q133" s="5"/>
-      <c r="R133" s="5"/>
+      <c r="B133" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C133" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D133" s="12"/>
+      <c r="E133" s="12"/>
+      <c r="F133" s="12"/>
+      <c r="G133" s="12"/>
+      <c r="H133" s="12"/>
+      <c r="I133" s="12"/>
+      <c r="J133" s="12"/>
+      <c r="K133" s="12"/>
+      <c r="L133" s="12"/>
+      <c r="M133" s="12"/>
+      <c r="N133" s="12"/>
+      <c r="O133" s="12"/>
+      <c r="P133" s="12"/>
+      <c r="Q133" s="12"/>
+      <c r="R133" s="12"/>
     </row>
     <row r="134" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B134" s="6"/>
-      <c r="C134" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D134" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E134" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F134" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G134" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H134" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I134" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J134" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K134" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L134" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="M134" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="N134" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O134" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P134" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q134" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="R134" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="B134" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C134" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D134" s="12"/>
+      <c r="E134" s="12"/>
+      <c r="F134" s="12"/>
+      <c r="G134" s="12"/>
+      <c r="H134" s="12"/>
+      <c r="I134" s="12"/>
+      <c r="J134" s="12"/>
+      <c r="K134" s="12"/>
+      <c r="L134" s="12"/>
+      <c r="M134" s="12"/>
+      <c r="N134" s="12"/>
+      <c r="O134" s="12"/>
+      <c r="P134" s="12"/>
+      <c r="Q134" s="12"/>
+      <c r="R134" s="12"/>
     </row>
     <row r="135" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B135" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C135" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="D135" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="E135" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="F135" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="S135" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="136" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B136" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="R136" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="S136" s="1" t="s">
-        <v>112</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="C135" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D135" s="12"/>
+      <c r="E135" s="12"/>
+      <c r="F135" s="12"/>
+      <c r="G135" s="12"/>
+      <c r="H135" s="12"/>
+      <c r="I135" s="12"/>
+      <c r="J135" s="12"/>
+      <c r="K135" s="12"/>
+      <c r="L135" s="12"/>
+      <c r="M135" s="12"/>
+      <c r="N135" s="12"/>
+      <c r="O135" s="12"/>
+      <c r="P135" s="12"/>
+      <c r="Q135" s="12"/>
+      <c r="R135" s="12"/>
+    </row>
+    <row r="137" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B137" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C137" s="5"/>
+      <c r="D137" s="5"/>
+      <c r="E137" s="5"/>
+      <c r="F137" s="5"/>
+      <c r="G137" s="5"/>
+      <c r="H137" s="5"/>
+      <c r="I137" s="5"/>
+      <c r="J137" s="5"/>
+      <c r="K137" s="5"/>
+      <c r="L137" s="5"/>
+      <c r="M137" s="5"/>
+      <c r="N137" s="5"/>
+      <c r="O137" s="5"/>
+      <c r="P137" s="5"/>
+      <c r="Q137" s="5"/>
+      <c r="R137" s="5"/>
     </row>
     <row r="138" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B138" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C138" s="5"/>
-      <c r="D138" s="5"/>
-      <c r="E138" s="5"/>
-      <c r="F138" s="5"/>
-      <c r="G138" s="5"/>
-      <c r="H138" s="5"/>
-      <c r="I138" s="5"/>
-      <c r="J138" s="5"/>
-      <c r="K138" s="5"/>
-      <c r="L138" s="5"/>
-      <c r="M138" s="5"/>
-      <c r="N138" s="5"/>
-      <c r="O138" s="5"/>
-      <c r="P138" s="5"/>
-      <c r="Q138" s="5"/>
-      <c r="R138" s="5"/>
+      <c r="B138" s="6"/>
+      <c r="C138" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D138" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E138" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F138" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G138" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H138" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I138" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J138" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K138" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L138" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M138" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="N138" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O138" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P138" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q138" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R138" s="7" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B139" s="6"/>
-      <c r="C139" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D139" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E139" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F139" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G139" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H139" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I139" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J139" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K139" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L139" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="M139" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="N139" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O139" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P139" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q139" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="R139" s="7" t="s">
-        <v>7</v>
+      <c r="B139" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D139" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="S139" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="T139" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="S140" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B141" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C141" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D141" s="10"/>
+      <c r="E141" s="10"/>
+      <c r="F141" s="10"/>
+      <c r="G141" s="10"/>
+      <c r="H141" s="10"/>
+      <c r="I141" s="10"/>
+      <c r="J141" s="10"/>
+      <c r="K141" s="10"/>
+      <c r="L141" s="10"/>
+      <c r="M141" s="10"/>
+      <c r="N141" s="10"/>
+      <c r="O141" s="10"/>
+      <c r="P141" s="10"/>
+      <c r="Q141" s="10"/>
+      <c r="R141" s="10"/>
+    </row>
+    <row r="142" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B142" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C142" s="10"/>
+      <c r="D142" s="10"/>
+      <c r="E142" s="10"/>
+      <c r="F142" s="10"/>
+      <c r="G142" s="10"/>
+      <c r="H142" s="10"/>
+      <c r="I142" s="10"/>
+      <c r="J142" s="10"/>
+      <c r="K142" s="10"/>
+      <c r="L142" s="10"/>
+      <c r="M142" s="10"/>
+      <c r="N142" s="10"/>
+      <c r="O142" s="10"/>
+      <c r="P142" s="10"/>
+      <c r="Q142" s="10"/>
+      <c r="R142" s="10"/>
+    </row>
+    <row r="144" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B144" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C144" s="5"/>
+      <c r="D144" s="5"/>
+      <c r="E144" s="5"/>
+      <c r="F144" s="5"/>
+      <c r="G144" s="5"/>
+      <c r="H144" s="5"/>
+      <c r="I144" s="5"/>
+      <c r="J144" s="5"/>
+      <c r="K144" s="5"/>
+      <c r="L144" s="5"/>
+      <c r="M144" s="5"/>
+      <c r="N144" s="5"/>
+      <c r="O144" s="5"/>
+      <c r="P144" s="5"/>
+      <c r="Q144" s="5"/>
+      <c r="R144" s="5"/>
+      <c r="S144" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B145" s="6"/>
+      <c r="C145" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D145" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E145" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F145" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G145" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H145" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I145" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J145" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K145" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L145" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M145" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="N145" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O145" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P145" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q145" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R145" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B146" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D146" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E146" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F146" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G146" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H146" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I146" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J146" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="K146" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L146" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="M146" s="14"/>
+      <c r="N146" s="14"/>
+      <c r="O146" s="14"/>
+      <c r="P146" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q146" s="14"/>
+      <c r="R146" s="14"/>
+    </row>
+    <row r="147" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B147" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D147" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E147" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F147" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G147" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H147" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I147" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J147" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="K147" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="L147" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M147" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="N147" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="O147" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P147" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q147" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="R147" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B148" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C148" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E148" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F148" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G148" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="H148" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="I148" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="J148" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="K148" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="L148" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="M148" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="N148" s="14"/>
+      <c r="O148" s="14"/>
+      <c r="P148" s="14"/>
+      <c r="Q148" s="14"/>
+      <c r="R148" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B150" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C150" s="5"/>
+      <c r="D150" s="5"/>
+      <c r="E150" s="5"/>
+      <c r="F150" s="5"/>
+      <c r="G150" s="5"/>
+      <c r="H150" s="5"/>
+      <c r="I150" s="5"/>
+      <c r="J150" s="5"/>
+      <c r="K150" s="5"/>
+      <c r="L150" s="5"/>
+      <c r="M150" s="5"/>
+      <c r="N150" s="5"/>
+      <c r="O150" s="5"/>
+      <c r="P150" s="5"/>
+      <c r="Q150" s="5"/>
+      <c r="R150" s="5"/>
+    </row>
+    <row r="151" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B151" s="6"/>
+      <c r="C151" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D151" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E151" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F151" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G151" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H151" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I151" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J151" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K151" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L151" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M151" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="N151" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O151" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P151" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q151" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R151" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B152" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C152" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E152" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F152" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="S152" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B153" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C140" s="16" t="s">
+      <c r="R153" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D140" s="3" t="s">
+      <c r="S153" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E140" s="3" t="s">
+    </row>
+    <row r="155" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B155" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="F140" s="3" t="s">
+      <c r="C155" s="5"/>
+      <c r="D155" s="5"/>
+      <c r="E155" s="5"/>
+      <c r="F155" s="5"/>
+      <c r="G155" s="5"/>
+      <c r="H155" s="5"/>
+      <c r="I155" s="5"/>
+      <c r="J155" s="5"/>
+      <c r="K155" s="5"/>
+      <c r="L155" s="5"/>
+      <c r="M155" s="5"/>
+      <c r="N155" s="5"/>
+      <c r="O155" s="5"/>
+      <c r="P155" s="5"/>
+      <c r="Q155" s="5"/>
+      <c r="R155" s="5"/>
+    </row>
+    <row r="156" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B156" s="6"/>
+      <c r="C156" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D156" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E156" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F156" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G156" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H156" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I156" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J156" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K156" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L156" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M156" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="N156" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O156" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P156" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q156" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R156" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B157" s="2" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B142" s="5" t="s">
+      <c r="C157" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="C142" s="5"/>
-      <c r="D142" s="5"/>
-      <c r="E142" s="5"/>
-      <c r="F142" s="5"/>
-      <c r="G142" s="5"/>
-      <c r="H142" s="5"/>
-      <c r="I142" s="5"/>
-      <c r="J142" s="5"/>
-      <c r="K142" s="5"/>
-      <c r="L142" s="5"/>
-      <c r="M142" s="5"/>
-      <c r="N142" s="5"/>
-      <c r="O142" s="5"/>
-      <c r="P142" s="5"/>
-      <c r="Q142" s="5"/>
-      <c r="R142" s="5"/>
-    </row>
-    <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B143" s="6"/>
-      <c r="C143" s="7" t="n">
+      <c r="D157" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E157" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F157" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B159" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C159" s="5"/>
+      <c r="D159" s="5"/>
+      <c r="E159" s="5"/>
+      <c r="F159" s="5"/>
+      <c r="G159" s="5"/>
+      <c r="H159" s="5"/>
+      <c r="I159" s="5"/>
+      <c r="J159" s="5"/>
+      <c r="K159" s="5"/>
+      <c r="L159" s="5"/>
+      <c r="M159" s="5"/>
+      <c r="N159" s="5"/>
+      <c r="O159" s="5"/>
+      <c r="P159" s="5"/>
+      <c r="Q159" s="5"/>
+      <c r="R159" s="5"/>
+    </row>
+    <row r="160" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B160" s="6"/>
+      <c r="C160" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D143" s="7" t="n">
+      <c r="D160" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E143" s="7" t="n">
+      <c r="E160" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F143" s="7" t="n">
+      <c r="F160" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G143" s="7" t="n">
+      <c r="G160" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="H143" s="7" t="n">
+      <c r="H160" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="I143" s="7" t="n">
+      <c r="I160" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="J143" s="7" t="n">
+      <c r="J160" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="K143" s="7" t="n">
+      <c r="K160" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="L143" s="7" t="n">
+      <c r="L160" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="M143" s="7" t="s">
+      <c r="M160" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="N143" s="7" t="s">
+      <c r="N160" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="O143" s="7" t="s">
+      <c r="O160" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="P143" s="7" t="s">
+      <c r="P160" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="Q143" s="7" t="s">
+      <c r="Q160" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="R143" s="7" t="s">
+      <c r="R160" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B144" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C144" s="3" t="n">
+    <row r="161" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B161" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C161" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D144" s="3" t="n">
+      <c r="D161" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E144" s="3" t="n">
+      <c r="E161" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F144" s="3" t="n">
+      <c r="F161" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G144" s="3" t="n">
+      <c r="G161" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H144" s="3" t="n">
+      <c r="H161" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="I144" s="3" t="n">
+      <c r="I161" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="J144" s="3" t="n">
+      <c r="J161" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="K144" s="3" t="n">
+      <c r="K161" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="L144" s="3" t="n">
+      <c r="L161" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="M144" s="3" t="n">
+      <c r="M161" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="N144" s="3" t="n">
+      <c r="N161" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="O144" s="3" t="n">
+      <c r="O161" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="P144" s="3" t="n">
+      <c r="P161" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="Q144" s="3" t="n">
+      <c r="Q161" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="R144" s="3" t="n">
+      <c r="R161" s="3" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B146" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="C146" s="5"/>
-      <c r="D146" s="5"/>
-      <c r="E146" s="5"/>
-      <c r="F146" s="5"/>
-      <c r="G146" s="5"/>
-      <c r="H146" s="5"/>
-      <c r="I146" s="5"/>
-      <c r="J146" s="5"/>
-      <c r="K146" s="5"/>
-      <c r="L146" s="5"/>
-      <c r="M146" s="5"/>
-      <c r="N146" s="5"/>
-      <c r="O146" s="5"/>
-      <c r="P146" s="5"/>
-      <c r="Q146" s="5"/>
-      <c r="R146" s="5"/>
-    </row>
-    <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B147" s="6"/>
-      <c r="C147" s="7" t="n">
+    <row r="163" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B163" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C163" s="5"/>
+      <c r="D163" s="5"/>
+      <c r="E163" s="5"/>
+      <c r="F163" s="5"/>
+      <c r="G163" s="5"/>
+      <c r="H163" s="5"/>
+      <c r="I163" s="5"/>
+      <c r="J163" s="5"/>
+      <c r="K163" s="5"/>
+      <c r="L163" s="5"/>
+      <c r="M163" s="5"/>
+      <c r="N163" s="5"/>
+      <c r="O163" s="5"/>
+      <c r="P163" s="5"/>
+      <c r="Q163" s="5"/>
+      <c r="R163" s="5"/>
+    </row>
+    <row r="164" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B164" s="6"/>
+      <c r="C164" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D147" s="7" t="n">
+      <c r="D164" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E147" s="7" t="n">
+      <c r="E164" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F147" s="7" t="n">
+      <c r="F164" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G147" s="7" t="n">
+      <c r="G164" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="H147" s="7" t="n">
+      <c r="H164" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="I147" s="7" t="n">
+      <c r="I164" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="J147" s="7" t="n">
+      <c r="J164" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="K147" s="7" t="n">
+      <c r="K164" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="L147" s="7" t="n">
+      <c r="L164" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="M147" s="7" t="s">
+      <c r="M164" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="N147" s="7" t="s">
+      <c r="N164" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="O147" s="7" t="s">
+      <c r="O164" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="P147" s="7" t="s">
+      <c r="P164" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="Q147" s="7" t="s">
+      <c r="Q164" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="R147" s="7" t="s">
+      <c r="R164" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B148" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="C148" s="16" t="n">
+    <row r="165" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B165" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C165" s="15" t="n">
         <v>-1</v>
       </c>
-      <c r="D148" s="3" t="n">
+      <c r="D165" s="3" t="n">
         <v>-2</v>
       </c>
-      <c r="E148" s="3" t="n">
+      <c r="E165" s="3" t="n">
         <v>-3</v>
       </c>
-      <c r="F148" s="3" t="n">
+      <c r="F165" s="3" t="n">
         <v>-4</v>
       </c>
-      <c r="G148" s="3" t="n">
+      <c r="G165" s="3" t="n">
         <v>-5</v>
       </c>
-      <c r="H148" s="3" t="n">
+      <c r="H165" s="3" t="n">
         <v>-6</v>
       </c>
-      <c r="I148" s="3" t="n">
+      <c r="I165" s="3" t="n">
         <v>-7</v>
       </c>
-      <c r="J148" s="3" t="n">
+      <c r="J165" s="3" t="n">
         <v>-8</v>
       </c>
-      <c r="K148" s="3" t="n">
+      <c r="K165" s="3" t="n">
         <v>-9</v>
       </c>
-      <c r="L148" s="3" t="n">
+      <c r="L165" s="3" t="n">
         <v>-10</v>
       </c>
-      <c r="M148" s="3" t="n">
+      <c r="M165" s="3" t="n">
         <v>-11</v>
       </c>
-      <c r="N148" s="3" t="n">
+      <c r="N165" s="3" t="n">
         <v>-12</v>
       </c>
-      <c r="O148" s="3" t="n">
+      <c r="O165" s="3" t="n">
         <v>-13</v>
       </c>
-      <c r="P148" s="3" t="n">
+      <c r="P165" s="3" t="n">
         <v>-14</v>
       </c>
-      <c r="Q148" s="3" t="n">
+      <c r="Q165" s="3" t="n">
         <v>-15</v>
       </c>
-      <c r="R148" s="3" t="n">
+      <c r="R165" s="3" t="n">
         <v>-16</v>
       </c>
-      <c r="S148" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B149" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C149" s="3" t="n">
+      <c r="S165" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B166" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C166" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D149" s="3" t="n">
+      <c r="D166" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E149" s="3" t="n">
+      <c r="E166" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F149" s="3" t="n">
+      <c r="F166" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G149" s="3" t="n">
+      <c r="G166" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H149" s="3" t="n">
+      <c r="H166" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="I149" s="3" t="n">
+      <c r="I166" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="J149" s="3" t="n">
+      <c r="J166" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="K149" s="3" t="n">
+      <c r="K166" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="L149" s="3" t="n">
+      <c r="L166" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="M149" s="3" t="n">
+      <c r="M166" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="N149" s="3" t="n">
+      <c r="N166" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="O149" s="3" t="n">
+      <c r="O166" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="P149" s="3" t="n">
+      <c r="P166" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="Q149" s="3" t="n">
+      <c r="Q166" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="R149" s="3" t="n">
+      <c r="R166" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="S149" s="1" t="s">
-        <v>125</v>
+      <c r="S166" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="A1:R1"/>
     <mergeCell ref="B3:R3"/>
     <mergeCell ref="C5:R10"/>
@@ -4608,27 +4935,28 @@
     <mergeCell ref="C21:R84"/>
     <mergeCell ref="C85:R86"/>
     <mergeCell ref="C87:R92"/>
-    <mergeCell ref="B103:R103"/>
-    <mergeCell ref="C105:R105"/>
-    <mergeCell ref="C106:R106"/>
-    <mergeCell ref="C107:R107"/>
-    <mergeCell ref="C108:R108"/>
-    <mergeCell ref="C109:R109"/>
-    <mergeCell ref="C110:R110"/>
-    <mergeCell ref="B112:R112"/>
-    <mergeCell ref="C113:R113"/>
-    <mergeCell ref="C114:R114"/>
-    <mergeCell ref="C115:R115"/>
-    <mergeCell ref="C116:R116"/>
-    <mergeCell ref="C117:R117"/>
-    <mergeCell ref="C118:R118"/>
+    <mergeCell ref="C101:R105"/>
     <mergeCell ref="B120:R120"/>
-    <mergeCell ref="C124:R125"/>
-    <mergeCell ref="B127:R127"/>
-    <mergeCell ref="B133:R133"/>
-    <mergeCell ref="B138:R138"/>
-    <mergeCell ref="B142:R142"/>
-    <mergeCell ref="B146:R146"/>
+    <mergeCell ref="C122:R122"/>
+    <mergeCell ref="C123:R123"/>
+    <mergeCell ref="C124:R124"/>
+    <mergeCell ref="C125:R125"/>
+    <mergeCell ref="C126:R126"/>
+    <mergeCell ref="C127:R127"/>
+    <mergeCell ref="B129:R129"/>
+    <mergeCell ref="C130:R130"/>
+    <mergeCell ref="C131:R131"/>
+    <mergeCell ref="C132:R132"/>
+    <mergeCell ref="C133:R133"/>
+    <mergeCell ref="C134:R134"/>
+    <mergeCell ref="C135:R135"/>
+    <mergeCell ref="B137:R137"/>
+    <mergeCell ref="C141:R142"/>
+    <mergeCell ref="B144:R144"/>
+    <mergeCell ref="B150:R150"/>
+    <mergeCell ref="B155:R155"/>
+    <mergeCell ref="B159:R159"/>
+    <mergeCell ref="B163:R163"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4646,16 +4974,16 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:R37"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15.4" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="3" style="1" width="4"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -4676,23 +5004,23 @@
       <c r="R1" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="17"/>
-      <c r="O3" s="17"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="17"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
     </row>
     <row r="5" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="6"/>
@@ -4749,364 +5077,364 @@
       <c r="B6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
+      <c r="C6" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
     </row>
     <row r="7" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
-      <c r="P7" s="19"/>
-      <c r="Q7" s="19"/>
-      <c r="R7" s="19"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-      <c r="I8" s="19"/>
-      <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
-      <c r="L8" s="19"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="19"/>
-      <c r="O8" s="19"/>
-      <c r="P8" s="19"/>
-      <c r="Q8" s="19"/>
-      <c r="R8" s="19"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="18"/>
+      <c r="N8" s="18"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="18"/>
+      <c r="Q8" s="18"/>
+      <c r="R8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="19"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="19"/>
-      <c r="N9" s="19"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="19"/>
-      <c r="Q9" s="19"/>
-      <c r="R9" s="19"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
+      <c r="R9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="19"/>
-      <c r="O10" s="19"/>
-      <c r="P10" s="19"/>
-      <c r="Q10" s="19"/>
-      <c r="R10" s="19"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="18"/>
+      <c r="Q10" s="18"/>
+      <c r="R10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="19"/>
-      <c r="N11" s="19"/>
-      <c r="O11" s="19"/>
-      <c r="P11" s="19"/>
-      <c r="Q11" s="19"/>
-      <c r="R11" s="19"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
+      <c r="L11" s="18"/>
+      <c r="M11" s="18"/>
+      <c r="N11" s="18"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="18"/>
+      <c r="Q11" s="18"/>
+      <c r="R11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
-      <c r="N12" s="19"/>
-      <c r="O12" s="19"/>
-      <c r="P12" s="19"/>
-      <c r="Q12" s="19"/>
-      <c r="R12" s="19"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="18"/>
+      <c r="M12" s="18"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="18"/>
+      <c r="Q12" s="18"/>
+      <c r="R12" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="19"/>
-      <c r="L13" s="19"/>
-      <c r="M13" s="19"/>
-      <c r="N13" s="19"/>
-      <c r="O13" s="19"/>
-      <c r="P13" s="19"/>
-      <c r="Q13" s="19"/>
-      <c r="R13" s="19"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="18"/>
+      <c r="M13" s="18"/>
+      <c r="N13" s="18"/>
+      <c r="O13" s="18"/>
+      <c r="P13" s="18"/>
+      <c r="Q13" s="18"/>
+      <c r="R13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="19"/>
-      <c r="M14" s="19"/>
-      <c r="N14" s="19"/>
-      <c r="O14" s="19"/>
-      <c r="P14" s="19"/>
-      <c r="Q14" s="19"/>
-      <c r="R14" s="19"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="18"/>
+      <c r="M14" s="18"/>
+      <c r="N14" s="18"/>
+      <c r="O14" s="18"/>
+      <c r="P14" s="18"/>
+      <c r="Q14" s="18"/>
+      <c r="R14" s="18"/>
     </row>
     <row r="15" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="19"/>
-      <c r="M15" s="19"/>
-      <c r="N15" s="19"/>
-      <c r="O15" s="19"/>
-      <c r="P15" s="19"/>
-      <c r="Q15" s="19"/>
-      <c r="R15" s="19"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
+      <c r="M15" s="18"/>
+      <c r="N15" s="18"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
+      <c r="R15" s="18"/>
     </row>
     <row r="16" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
-      <c r="O16" s="19"/>
-      <c r="P16" s="19"/>
-      <c r="Q16" s="19"/>
-      <c r="R16" s="19"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="18"/>
+      <c r="M16" s="18"/>
+      <c r="N16" s="18"/>
+      <c r="O16" s="18"/>
+      <c r="P16" s="18"/>
+      <c r="Q16" s="18"/>
+      <c r="R16" s="18"/>
     </row>
     <row r="17" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="19"/>
-      <c r="O17" s="19"/>
-      <c r="P17" s="19"/>
-      <c r="Q17" s="19"/>
-      <c r="R17" s="19"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="18"/>
+      <c r="M17" s="18"/>
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="18"/>
+      <c r="R17" s="18"/>
     </row>
     <row r="18" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
-      <c r="O18" s="19"/>
-      <c r="P18" s="19"/>
-      <c r="Q18" s="19"/>
-      <c r="R18" s="19"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="18"/>
+      <c r="P18" s="18"/>
+      <c r="Q18" s="18"/>
+      <c r="R18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
-      <c r="O19" s="19"/>
-      <c r="P19" s="19"/>
-      <c r="Q19" s="19"/>
-      <c r="R19" s="19"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
+      <c r="L19" s="18"/>
+      <c r="M19" s="18"/>
+      <c r="N19" s="18"/>
+      <c r="O19" s="18"/>
+      <c r="P19" s="18"/>
+      <c r="Q19" s="18"/>
+      <c r="R19" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
-      <c r="P20" s="19"/>
-      <c r="Q20" s="19"/>
-      <c r="R20" s="19"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="18"/>
+      <c r="M20" s="18"/>
+      <c r="N20" s="18"/>
+      <c r="O20" s="18"/>
+      <c r="P20" s="18"/>
+      <c r="Q20" s="18"/>
+      <c r="R20" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="19"/>
-      <c r="O21" s="19"/>
-      <c r="P21" s="19"/>
-      <c r="Q21" s="19"/>
-      <c r="R21" s="19"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18"/>
+      <c r="L21" s="18"/>
+      <c r="M21" s="18"/>
+      <c r="N21" s="18"/>
+      <c r="O21" s="18"/>
+      <c r="P21" s="18"/>
+      <c r="Q21" s="18"/>
+      <c r="R21" s="18"/>
     </row>
     <row r="22" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="19"/>
-      <c r="O22" s="19"/>
-      <c r="P22" s="19"/>
-      <c r="Q22" s="19"/>
-      <c r="R22" s="19"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
+      <c r="L22" s="18"/>
+      <c r="M22" s="18"/>
+      <c r="N22" s="18"/>
+      <c r="O22" s="18"/>
+      <c r="P22" s="18"/>
+      <c r="Q22" s="18"/>
+      <c r="R22" s="18"/>
     </row>
     <row r="23" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
@@ -5126,7 +5454,7 @@
     </row>
     <row r="24" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -5147,7 +5475,7 @@
     </row>
     <row r="25" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -5167,8 +5495,8 @@
       <c r="R25" s="10"/>
     </row>
     <row r="26" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="20" t="s">
-        <v>132</v>
+      <c r="B26" s="19" t="s">
+        <v>36</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
@@ -5189,7 +5517,7 @@
     </row>
     <row r="27" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
@@ -5210,7 +5538,7 @@
     </row>
     <row r="28" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
@@ -5231,7 +5559,7 @@
     </row>
     <row r="29" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
@@ -5251,148 +5579,148 @@
       <c r="R29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="19"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="19"/>
-      <c r="N30" s="19"/>
-      <c r="O30" s="19"/>
-      <c r="P30" s="19"/>
-      <c r="Q30" s="19"/>
-      <c r="R30" s="19"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="18"/>
+      <c r="L30" s="18"/>
+      <c r="M30" s="18"/>
+      <c r="N30" s="18"/>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
     </row>
     <row r="31" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="19"/>
-      <c r="J31" s="19"/>
-      <c r="K31" s="19"/>
-      <c r="L31" s="19"/>
-      <c r="M31" s="19"/>
-      <c r="N31" s="19"/>
-      <c r="O31" s="19"/>
-      <c r="P31" s="19"/>
-      <c r="Q31" s="19"/>
-      <c r="R31" s="19"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+      <c r="I31" s="18"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="18"/>
+      <c r="L31" s="18"/>
+      <c r="M31" s="18"/>
+      <c r="N31" s="18"/>
+      <c r="O31" s="18"/>
+      <c r="P31" s="18"/>
+      <c r="Q31" s="18"/>
+      <c r="R31" s="18"/>
     </row>
     <row r="32" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="19"/>
-      <c r="J32" s="19"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="19"/>
-      <c r="N32" s="19"/>
-      <c r="O32" s="19"/>
-      <c r="P32" s="19"/>
-      <c r="Q32" s="19"/>
-      <c r="R32" s="19"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="18"/>
+      <c r="L32" s="18"/>
+      <c r="M32" s="18"/>
+      <c r="N32" s="18"/>
+      <c r="O32" s="18"/>
+      <c r="P32" s="18"/>
+      <c r="Q32" s="18"/>
+      <c r="R32" s="18"/>
     </row>
     <row r="33" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="19"/>
-      <c r="L33" s="19"/>
-      <c r="M33" s="19"/>
-      <c r="N33" s="19"/>
-      <c r="O33" s="19"/>
-      <c r="P33" s="19"/>
-      <c r="Q33" s="19"/>
-      <c r="R33" s="19"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="18"/>
+      <c r="L33" s="18"/>
+      <c r="M33" s="18"/>
+      <c r="N33" s="18"/>
+      <c r="O33" s="18"/>
+      <c r="P33" s="18"/>
+      <c r="Q33" s="18"/>
+      <c r="R33" s="18"/>
     </row>
     <row r="34" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19"/>
-      <c r="J34" s="19"/>
-      <c r="K34" s="19"/>
-      <c r="L34" s="19"/>
-      <c r="M34" s="19"/>
-      <c r="N34" s="19"/>
-      <c r="O34" s="19"/>
-      <c r="P34" s="19"/>
-      <c r="Q34" s="19"/>
-      <c r="R34" s="19"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
+      <c r="J34" s="18"/>
+      <c r="K34" s="18"/>
+      <c r="L34" s="18"/>
+      <c r="M34" s="18"/>
+      <c r="N34" s="18"/>
+      <c r="O34" s="18"/>
+      <c r="P34" s="18"/>
+      <c r="Q34" s="18"/>
+      <c r="R34" s="18"/>
     </row>
     <row r="35" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="19"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="19"/>
-      <c r="J35" s="19"/>
-      <c r="K35" s="19"/>
-      <c r="L35" s="19"/>
-      <c r="M35" s="19"/>
-      <c r="N35" s="19"/>
-      <c r="O35" s="19"/>
-      <c r="P35" s="19"/>
-      <c r="Q35" s="19"/>
-      <c r="R35" s="19"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
+      <c r="J35" s="18"/>
+      <c r="K35" s="18"/>
+      <c r="L35" s="18"/>
+      <c r="M35" s="18"/>
+      <c r="N35" s="18"/>
+      <c r="O35" s="18"/>
+      <c r="P35" s="18"/>
+      <c r="Q35" s="18"/>
+      <c r="R35" s="18"/>
     </row>
     <row r="36" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="19"/>
-      <c r="J36" s="19"/>
-      <c r="K36" s="19"/>
-      <c r="L36" s="19"/>
-      <c r="M36" s="19"/>
-      <c r="N36" s="19"/>
-      <c r="O36" s="19"/>
-      <c r="P36" s="19"/>
-      <c r="Q36" s="19"/>
-      <c r="R36" s="19"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="18"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="18"/>
+      <c r="L36" s="18"/>
+      <c r="M36" s="18"/>
+      <c r="N36" s="18"/>
+      <c r="O36" s="18"/>
+      <c r="P36" s="18"/>
+      <c r="Q36" s="18"/>
+      <c r="R36" s="18"/>
     </row>
     <row r="37" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="19"/>
-      <c r="J37" s="19"/>
-      <c r="K37" s="19"/>
-      <c r="L37" s="19"/>
-      <c r="M37" s="19"/>
-      <c r="N37" s="19"/>
-      <c r="O37" s="19"/>
-      <c r="P37" s="19"/>
-      <c r="Q37" s="19"/>
-      <c r="R37" s="19"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="18"/>
+      <c r="J37" s="18"/>
+      <c r="K37" s="18"/>
+      <c r="L37" s="18"/>
+      <c r="M37" s="18"/>
+      <c r="N37" s="18"/>
+      <c r="O37" s="18"/>
+      <c r="P37" s="18"/>
+      <c r="Q37" s="18"/>
+      <c r="R37" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Full Cyrillic, CyrlExtA/B support (enables church slavonic)
</commit_message>
<xml_diff>
--- a/PUA_allocation_chart.xlsx
+++ b/PUA_allocation_chart.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="142">
   <si>
     <t xml:space="preserve">PUA Allocation Chart U+Fxxxx</t>
   </si>
@@ -236,10 +236,19 @@
     <t xml:space="preserve">Pm</t>
   </si>
   <si>
+    <t xml:space="preserve">ꙮ</t>
+  </si>
+  <si>
     <t xml:space="preserve">Placeholder Majuscule</t>
   </si>
   <si>
     <t xml:space="preserve">Placeholder Miniscule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seraphimi left</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seraphimi right</t>
   </si>
   <si>
     <t xml:space="preserve">FFE1</t>
@@ -944,7 +953,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U166"/>
+  <dimension ref="A1:V166"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15.4" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.71"/>
@@ -4146,30 +4155,42 @@
       <c r="D139" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="E139" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F139" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="S139" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="T139" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
+      </c>
+      <c r="U139" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="V139" s="0" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="S140" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C141" s="10" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D141" s="10"/>
       <c r="E141" s="10"/>
@@ -4189,7 +4210,7 @@
     </row>
     <row r="142" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B142" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C142" s="10"/>
       <c r="D142" s="10"/>
@@ -4210,7 +4231,7 @@
     </row>
     <row r="144" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B144" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C144" s="5"/>
       <c r="D144" s="5"/>
@@ -4229,7 +4250,7 @@
       <c r="Q144" s="5"/>
       <c r="R144" s="5"/>
       <c r="S144" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4285,7 +4306,7 @@
     </row>
     <row r="146" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B146" s="2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C146" s="3" t="n">
         <v>0</v>
@@ -4321,17 +4342,17 @@
       <c r="N146" s="14"/>
       <c r="O146" s="14"/>
       <c r="P146" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="Q146" s="14"/>
       <c r="R146" s="14"/>
     </row>
     <row r="147" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B147" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>2</v>
@@ -4352,81 +4373,81 @@
         <v>7</v>
       </c>
       <c r="J147" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="K147" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="L147" s="3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="M147" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="N147" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="O147" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="P147" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="Q147" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="R147" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E148" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G148" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="I148" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="J148" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="K148" s="3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="L148" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="M148" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="N148" s="14"/>
       <c r="O148" s="14"/>
       <c r="P148" s="14"/>
       <c r="Q148" s="14"/>
       <c r="R148" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="5" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C150" s="5"/>
       <c r="D150" s="5"/>
@@ -4498,38 +4519,38 @@
     </row>
     <row r="152" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E152" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F152" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="S152" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B153" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="R153" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="S153" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B155" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C155" s="5"/>
       <c r="D155" s="5"/>
@@ -4601,24 +4622,24 @@
     </row>
     <row r="157" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B157" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C157" s="15" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E157" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F157" s="3" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B159" s="5" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C159" s="5"/>
       <c r="D159" s="5"/>
@@ -4690,7 +4711,7 @@
     </row>
     <row r="161" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B161" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C161" s="3" t="n">
         <v>1</v>
@@ -4743,7 +4764,7 @@
     </row>
     <row r="163" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B163" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C163" s="5"/>
       <c r="D163" s="5"/>
@@ -4815,7 +4836,7 @@
     </row>
     <row r="165" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B165" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C165" s="15" t="n">
         <v>-1</v>
@@ -4866,12 +4887,12 @@
         <v>-16</v>
       </c>
       <c r="S165" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C166" s="3" t="n">
         <v>1</v>
@@ -4922,7 +4943,7 @@
         <v>16</v>
       </c>
       <c r="S166" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -4983,7 +5004,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -5078,7 +5099,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D6" s="17"/>
       <c r="E6" s="17"/>
@@ -5431,10 +5452,10 @@
     </row>
     <row r="23" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
@@ -5454,7 +5475,7 @@
     </row>
     <row r="24" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -5475,7 +5496,7 @@
     </row>
     <row r="25" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -5517,7 +5538,7 @@
     </row>
     <row r="27" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
@@ -5538,7 +5559,7 @@
     </row>
     <row r="28" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
@@ -5559,7 +5580,7 @@
     </row>
     <row r="29" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>

</xml_diff>

<commit_message>
OTF hangul base addr remap
</commit_message>
<xml_diff>
--- a/PUA_allocation_chart.xlsx
+++ b/PUA_allocation_chart.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="140">
   <si>
     <t xml:space="preserve">PUA Allocation Chart U+Fxxxx</t>
   </si>
@@ -128,316 +128,310 @@
     <t xml:space="preserve">Codestyle ASCII Variants</t>
   </si>
   <si>
-    <t xml:space="preserve">Hangul Jamo Variants</t>
+    <t xml:space="preserve">Small ASCII Characters for Super/Subscript Composition Used Internally</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Todo: these codes may be moved outside of Unicode or use its own codespace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASCII Subscripts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Also requires Unicode-to-PUA conversion table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F806</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASCII Superscripts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F80C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematics Blackboard Bold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F812</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematics Fraktur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F818</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematics Cursive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F81E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mathematics Bold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typewriter Input Character Codes (Used By Terrarum Typewriter project)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F900</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typewriter Intl Qwerty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F910</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typewriter Intl Colemak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F920</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typewriter Intl Dvorak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F930</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typewriter Fr Bépo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F9**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typewriter ……</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FA00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typewriter Ko 3set-390</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal Symbols</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFE0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ꙮ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placeholder Majuscule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placeholder Miniscule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seraphimi left</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seraphimi right</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFE1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ꞱM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superscript Falsum Trademark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFE2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IPA Intonation Graph Fragments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFE3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal Object Identifiers (used by b.TᴇX Typesetter)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format: OBJ &lt;identifier glyphs&gt; ID-END</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFF7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFF8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFF9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID-END</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rich Text Modifiers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RBM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RBS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ruby Master; Ruby Slave; Superscript; Subscript</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFFB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">END</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAG END closes current tag, that is, works as '}' in LaTeX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charset Overrides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFFC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Default</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CODE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typesetting Placeholders (used by b.TᴇX Typesetter)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFFD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typesetting Glues (used by b.TᴇX Typesetter)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFFE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tight spaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loose spaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PUA Allocation Chart U+10xxxx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disable color code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTE: OTF version of the font uses U+100000..10187F for Hangul Jamo variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colour code U+10Fxxx in RGB order (LSB == Blue)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F02</t>
   </si>
   <si>
     <t xml:space="preserve">…</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F1E6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F1E7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small ASCII Characters for Super/Subscript Composition Used Internally</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Todo: these codes may be moved outside of Unicode or use its own codespace</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F800</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASCII Subscripts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Also requires Unicode-to-PUA conversion table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F806</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASCII Superscripts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F80C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mathematics Blackboard Bold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F812</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mathematics Fraktur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F818</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mathematics Cursive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F81E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mathematics Bold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typewriter Input Character Codes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F900</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typewriter Intl Qwerty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F910</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typewriter Intl Colemak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F920</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typewriter Intl Dvorak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F930</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typewriter Fr Bépo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F9**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typewriter ……</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FA00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typewriter Ko 3set-390</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internal Symbols</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFE0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ꙮ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placeholder Majuscule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placeholder Miniscule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seraphimi left</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seraphimi right</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFE1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ꞱM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Superscript Falsum Trademark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFE2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IPA Intonation Graph Fragments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFE3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internal Object Identifiers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format: OBJ &lt;identifier glyphs&gt; ID-END</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFF7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFF8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFF9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID-END</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rich Text Modifiers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFFA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RBM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RBS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ruby Master; Ruby Slave; Superscript; Subscript</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFFB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">END</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TAG END closes current tag, that is, works as '}' in LaTeX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charset Overrides</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFFC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Default</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CODE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typesetting Placeholders</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFFD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typesetting Glues</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFFE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tight spaces</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FFFF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loose spaces</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PUA Allocation Chart U+10xxxx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disable color code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colour code U+10Fxxx in RGB order (LSB == Blue)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F02</t>
   </si>
   <si>
     <t xml:space="preserve">FFD</t>
@@ -953,7 +947,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V166"/>
+  <dimension ref="A1:V1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15.4" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.71"/>
@@ -3356,1598 +3350,1341 @@
       <c r="R100" s="11"/>
     </row>
     <row r="101" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B101" s="2" t="str">
-        <f aca="false">"F06"&amp;RIGHT(B85,1)</f>
-        <v>F060</v>
-      </c>
-      <c r="C101" s="10" t="s">
+      <c r="C101" s="11"/>
+      <c r="D101" s="11"/>
+      <c r="E101" s="11"/>
+      <c r="F101" s="11"/>
+      <c r="G101" s="11"/>
+      <c r="H101" s="11"/>
+      <c r="I101" s="11"/>
+      <c r="J101" s="11"/>
+      <c r="K101" s="11"/>
+      <c r="L101" s="11"/>
+      <c r="M101" s="11"/>
+      <c r="N101" s="11"/>
+      <c r="O101" s="11"/>
+      <c r="P101" s="11"/>
+      <c r="Q101" s="11"/>
+      <c r="R101" s="11"/>
+    </row>
+    <row r="102" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C102" s="11"/>
+      <c r="D102" s="11"/>
+      <c r="E102" s="11"/>
+      <c r="F102" s="11"/>
+      <c r="G102" s="11"/>
+      <c r="H102" s="11"/>
+      <c r="I102" s="11"/>
+      <c r="J102" s="11"/>
+      <c r="K102" s="11"/>
+      <c r="L102" s="11"/>
+      <c r="M102" s="11"/>
+      <c r="N102" s="11"/>
+      <c r="O102" s="11"/>
+      <c r="P102" s="11"/>
+      <c r="Q102" s="11"/>
+      <c r="R102" s="11"/>
+    </row>
+    <row r="103" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C103" s="11"/>
+      <c r="D103" s="11"/>
+      <c r="E103" s="11"/>
+      <c r="F103" s="11"/>
+      <c r="G103" s="11"/>
+      <c r="H103" s="11"/>
+      <c r="I103" s="11"/>
+      <c r="J103" s="11"/>
+      <c r="K103" s="11"/>
+      <c r="L103" s="11"/>
+      <c r="M103" s="11"/>
+      <c r="N103" s="11"/>
+      <c r="O103" s="11"/>
+      <c r="P103" s="11"/>
+      <c r="Q103" s="11"/>
+      <c r="R103" s="11"/>
+    </row>
+    <row r="104" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C104" s="11"/>
+      <c r="D104" s="11"/>
+      <c r="E104" s="11"/>
+      <c r="F104" s="11"/>
+      <c r="G104" s="11"/>
+      <c r="H104" s="11"/>
+      <c r="I104" s="11"/>
+      <c r="J104" s="11"/>
+      <c r="K104" s="11"/>
+      <c r="L104" s="11"/>
+      <c r="M104" s="11"/>
+      <c r="N104" s="11"/>
+      <c r="O104" s="11"/>
+      <c r="P104" s="11"/>
+      <c r="Q104" s="11"/>
+      <c r="R104" s="11"/>
+    </row>
+    <row r="106" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B106" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D101" s="10"/>
-      <c r="E101" s="10"/>
-      <c r="F101" s="10"/>
-      <c r="G101" s="10"/>
-      <c r="H101" s="10"/>
-      <c r="I101" s="10"/>
-      <c r="J101" s="10"/>
-      <c r="K101" s="10"/>
-      <c r="L101" s="10"/>
-      <c r="M101" s="10"/>
-      <c r="N101" s="10"/>
-      <c r="O101" s="10"/>
-      <c r="P101" s="10"/>
-      <c r="Q101" s="10"/>
-      <c r="R101" s="10"/>
-    </row>
-    <row r="102" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B102" s="2" t="str">
-        <f aca="false">"F06"&amp;RIGHT(B86,1)</f>
-        <v>F061</v>
-      </c>
-      <c r="C102" s="10"/>
-      <c r="D102" s="10"/>
-      <c r="E102" s="10"/>
-      <c r="F102" s="10"/>
-      <c r="G102" s="10"/>
-      <c r="H102" s="10"/>
-      <c r="I102" s="10"/>
-      <c r="J102" s="10"/>
-      <c r="K102" s="10"/>
-      <c r="L102" s="10"/>
-      <c r="M102" s="10"/>
-      <c r="N102" s="10"/>
-      <c r="O102" s="10"/>
-      <c r="P102" s="10"/>
-      <c r="Q102" s="10"/>
-      <c r="R102" s="10"/>
-    </row>
-    <row r="103" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B103" s="2" t="s">
+      <c r="C106" s="5"/>
+      <c r="D106" s="5"/>
+      <c r="E106" s="5"/>
+      <c r="F106" s="5"/>
+      <c r="G106" s="5"/>
+      <c r="H106" s="5"/>
+      <c r="I106" s="5"/>
+      <c r="J106" s="5"/>
+      <c r="K106" s="5"/>
+      <c r="L106" s="5"/>
+      <c r="M106" s="5"/>
+      <c r="N106" s="5"/>
+      <c r="O106" s="5"/>
+      <c r="P106" s="5"/>
+      <c r="Q106" s="5"/>
+      <c r="R106" s="5"/>
+      <c r="S106" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C103" s="10"/>
-      <c r="D103" s="10"/>
-      <c r="E103" s="10"/>
-      <c r="F103" s="10"/>
-      <c r="G103" s="10"/>
-      <c r="H103" s="10"/>
-      <c r="I103" s="10"/>
-      <c r="J103" s="10"/>
-      <c r="K103" s="10"/>
-      <c r="L103" s="10"/>
-      <c r="M103" s="10"/>
-      <c r="N103" s="10"/>
-      <c r="O103" s="10"/>
-      <c r="P103" s="10"/>
-      <c r="Q103" s="10"/>
-      <c r="R103" s="10"/>
-    </row>
-    <row r="104" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B104" s="2" t="s">
+    </row>
+    <row r="107" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B107" s="6"/>
+      <c r="C107" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F107" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G107" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H107" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I107" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J107" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K107" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L107" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M107" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="N107" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O107" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P107" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q107" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R107" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B108" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C104" s="10"/>
-      <c r="D104" s="10"/>
-      <c r="E104" s="10"/>
-      <c r="F104" s="10"/>
-      <c r="G104" s="10"/>
-      <c r="H104" s="10"/>
-      <c r="I104" s="10"/>
-      <c r="J104" s="10"/>
-      <c r="K104" s="10"/>
-      <c r="L104" s="10"/>
-      <c r="M104" s="10"/>
-      <c r="N104" s="10"/>
-      <c r="O104" s="10"/>
-      <c r="P104" s="10"/>
-      <c r="Q104" s="10"/>
-      <c r="R104" s="10"/>
-    </row>
-    <row r="105" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B105" s="2" t="s">
+      <c r="C108" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C105" s="10"/>
-      <c r="D105" s="10"/>
-      <c r="E105" s="10"/>
-      <c r="F105" s="10"/>
-      <c r="G105" s="10"/>
-      <c r="H105" s="10"/>
-      <c r="I105" s="10"/>
-      <c r="J105" s="10"/>
-      <c r="K105" s="10"/>
-      <c r="L105" s="10"/>
-      <c r="M105" s="10"/>
-      <c r="N105" s="10"/>
-      <c r="O105" s="10"/>
-      <c r="P105" s="10"/>
-      <c r="Q105" s="10"/>
-      <c r="R105" s="10"/>
-    </row>
-    <row r="106" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C106" s="11"/>
-      <c r="D106" s="11"/>
-      <c r="E106" s="11"/>
-      <c r="F106" s="11"/>
-      <c r="G106" s="11"/>
-      <c r="H106" s="11"/>
-      <c r="I106" s="11"/>
-      <c r="J106" s="11"/>
-      <c r="K106" s="11"/>
-      <c r="L106" s="11"/>
-      <c r="M106" s="11"/>
-      <c r="N106" s="11"/>
-      <c r="O106" s="11"/>
-      <c r="P106" s="11"/>
-      <c r="Q106" s="11"/>
-      <c r="R106" s="11"/>
-    </row>
-    <row r="107" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C107" s="11"/>
-      <c r="D107" s="11"/>
-      <c r="E107" s="11"/>
-      <c r="F107" s="11"/>
-      <c r="G107" s="11"/>
-      <c r="H107" s="11"/>
-      <c r="I107" s="11"/>
-      <c r="J107" s="11"/>
-      <c r="K107" s="11"/>
-      <c r="L107" s="11"/>
-      <c r="M107" s="11"/>
-      <c r="N107" s="11"/>
-      <c r="O107" s="11"/>
-      <c r="P107" s="11"/>
-      <c r="Q107" s="11"/>
-      <c r="R107" s="11"/>
-    </row>
-    <row r="108" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C108" s="11"/>
-      <c r="D108" s="11"/>
-      <c r="E108" s="11"/>
-      <c r="F108" s="11"/>
-      <c r="G108" s="11"/>
-      <c r="H108" s="11"/>
-      <c r="I108" s="11"/>
-      <c r="J108" s="11"/>
-      <c r="K108" s="11"/>
-      <c r="L108" s="11"/>
-      <c r="M108" s="11"/>
-      <c r="N108" s="11"/>
-      <c r="O108" s="11"/>
-      <c r="P108" s="11"/>
-      <c r="Q108" s="11"/>
-      <c r="R108" s="11"/>
+      <c r="D108" s="12"/>
+      <c r="E108" s="12"/>
+      <c r="F108" s="12"/>
+      <c r="G108" s="12"/>
+      <c r="H108" s="12"/>
+      <c r="I108" s="12"/>
+      <c r="J108" s="12"/>
+      <c r="K108" s="12"/>
+      <c r="L108" s="12"/>
+      <c r="M108" s="12"/>
+      <c r="N108" s="12"/>
+      <c r="O108" s="12"/>
+      <c r="P108" s="12"/>
+      <c r="Q108" s="12"/>
+      <c r="R108" s="12"/>
+      <c r="S108" s="13" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C109" s="11"/>
-      <c r="D109" s="11"/>
-      <c r="E109" s="11"/>
-      <c r="F109" s="11"/>
-      <c r="G109" s="11"/>
-      <c r="H109" s="11"/>
-      <c r="I109" s="11"/>
-      <c r="J109" s="11"/>
-      <c r="K109" s="11"/>
-      <c r="L109" s="11"/>
-      <c r="M109" s="11"/>
-      <c r="N109" s="11"/>
-      <c r="O109" s="11"/>
-      <c r="P109" s="11"/>
-      <c r="Q109" s="11"/>
-      <c r="R109" s="11"/>
+      <c r="B109" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C109" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D109" s="12"/>
+      <c r="E109" s="12"/>
+      <c r="F109" s="12"/>
+      <c r="G109" s="12"/>
+      <c r="H109" s="12"/>
+      <c r="I109" s="12"/>
+      <c r="J109" s="12"/>
+      <c r="K109" s="12"/>
+      <c r="L109" s="12"/>
+      <c r="M109" s="12"/>
+      <c r="N109" s="12"/>
+      <c r="O109" s="12"/>
+      <c r="P109" s="12"/>
+      <c r="Q109" s="12"/>
+      <c r="R109" s="12"/>
     </row>
     <row r="110" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C110" s="11"/>
-      <c r="D110" s="11"/>
-      <c r="E110" s="11"/>
-      <c r="F110" s="11"/>
-      <c r="G110" s="11"/>
-      <c r="H110" s="11"/>
-      <c r="I110" s="11"/>
-      <c r="J110" s="11"/>
-      <c r="K110" s="11"/>
-      <c r="L110" s="11"/>
-      <c r="M110" s="11"/>
-      <c r="N110" s="11"/>
-      <c r="O110" s="11"/>
-      <c r="P110" s="11"/>
-      <c r="Q110" s="11"/>
-      <c r="R110" s="11"/>
+      <c r="B110" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C110" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D110" s="12"/>
+      <c r="E110" s="12"/>
+      <c r="F110" s="12"/>
+      <c r="G110" s="12"/>
+      <c r="H110" s="12"/>
+      <c r="I110" s="12"/>
+      <c r="J110" s="12"/>
+      <c r="K110" s="12"/>
+      <c r="L110" s="12"/>
+      <c r="M110" s="12"/>
+      <c r="N110" s="12"/>
+      <c r="O110" s="12"/>
+      <c r="P110" s="12"/>
+      <c r="Q110" s="12"/>
+      <c r="R110" s="12"/>
     </row>
     <row r="111" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C111" s="11"/>
-      <c r="D111" s="11"/>
-      <c r="E111" s="11"/>
-      <c r="F111" s="11"/>
-      <c r="G111" s="11"/>
-      <c r="H111" s="11"/>
-      <c r="I111" s="11"/>
-      <c r="J111" s="11"/>
-      <c r="K111" s="11"/>
-      <c r="L111" s="11"/>
-      <c r="M111" s="11"/>
-      <c r="N111" s="11"/>
-      <c r="O111" s="11"/>
-      <c r="P111" s="11"/>
-      <c r="Q111" s="11"/>
-      <c r="R111" s="11"/>
+      <c r="B111" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C111" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D111" s="12"/>
+      <c r="E111" s="12"/>
+      <c r="F111" s="12"/>
+      <c r="G111" s="12"/>
+      <c r="H111" s="12"/>
+      <c r="I111" s="12"/>
+      <c r="J111" s="12"/>
+      <c r="K111" s="12"/>
+      <c r="L111" s="12"/>
+      <c r="M111" s="12"/>
+      <c r="N111" s="12"/>
+      <c r="O111" s="12"/>
+      <c r="P111" s="12"/>
+      <c r="Q111" s="12"/>
+      <c r="R111" s="12"/>
     </row>
     <row r="112" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C112" s="11"/>
-      <c r="D112" s="11"/>
-      <c r="E112" s="11"/>
-      <c r="F112" s="11"/>
-      <c r="G112" s="11"/>
-      <c r="H112" s="11"/>
-      <c r="I112" s="11"/>
-      <c r="J112" s="11"/>
-      <c r="K112" s="11"/>
-      <c r="L112" s="11"/>
-      <c r="M112" s="11"/>
-      <c r="N112" s="11"/>
-      <c r="O112" s="11"/>
-      <c r="P112" s="11"/>
-      <c r="Q112" s="11"/>
-      <c r="R112" s="11"/>
+      <c r="B112" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C112" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D112" s="12"/>
+      <c r="E112" s="12"/>
+      <c r="F112" s="12"/>
+      <c r="G112" s="12"/>
+      <c r="H112" s="12"/>
+      <c r="I112" s="12"/>
+      <c r="J112" s="12"/>
+      <c r="K112" s="12"/>
+      <c r="L112" s="12"/>
+      <c r="M112" s="12"/>
+      <c r="N112" s="12"/>
+      <c r="O112" s="12"/>
+      <c r="P112" s="12"/>
+      <c r="Q112" s="12"/>
+      <c r="R112" s="12"/>
     </row>
     <row r="113" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C113" s="11"/>
-      <c r="D113" s="11"/>
-      <c r="E113" s="11"/>
-      <c r="F113" s="11"/>
-      <c r="G113" s="11"/>
-      <c r="H113" s="11"/>
-      <c r="I113" s="11"/>
-      <c r="J113" s="11"/>
-      <c r="K113" s="11"/>
-      <c r="L113" s="11"/>
-      <c r="M113" s="11"/>
-      <c r="N113" s="11"/>
-      <c r="O113" s="11"/>
-      <c r="P113" s="11"/>
-      <c r="Q113" s="11"/>
-      <c r="R113" s="11"/>
-    </row>
-    <row r="114" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C114" s="11"/>
-      <c r="D114" s="11"/>
-      <c r="E114" s="11"/>
-      <c r="F114" s="11"/>
-      <c r="G114" s="11"/>
-      <c r="H114" s="11"/>
-      <c r="I114" s="11"/>
-      <c r="J114" s="11"/>
-      <c r="K114" s="11"/>
-      <c r="L114" s="11"/>
-      <c r="M114" s="11"/>
-      <c r="N114" s="11"/>
-      <c r="O114" s="11"/>
-      <c r="P114" s="11"/>
-      <c r="Q114" s="11"/>
-      <c r="R114" s="11"/>
+      <c r="B113" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C113" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D113" s="12"/>
+      <c r="E113" s="12"/>
+      <c r="F113" s="12"/>
+      <c r="G113" s="12"/>
+      <c r="H113" s="12"/>
+      <c r="I113" s="12"/>
+      <c r="J113" s="12"/>
+      <c r="K113" s="12"/>
+      <c r="L113" s="12"/>
+      <c r="M113" s="12"/>
+      <c r="N113" s="12"/>
+      <c r="O113" s="12"/>
+      <c r="P113" s="12"/>
+      <c r="Q113" s="12"/>
+      <c r="R113" s="12"/>
     </row>
     <row r="115" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C115" s="11"/>
-      <c r="D115" s="11"/>
-      <c r="E115" s="11"/>
-      <c r="F115" s="11"/>
-      <c r="G115" s="11"/>
-      <c r="H115" s="11"/>
-      <c r="I115" s="11"/>
-      <c r="J115" s="11"/>
-      <c r="K115" s="11"/>
-      <c r="L115" s="11"/>
-      <c r="M115" s="11"/>
-      <c r="N115" s="11"/>
-      <c r="O115" s="11"/>
-      <c r="P115" s="11"/>
-      <c r="Q115" s="11"/>
-      <c r="R115" s="11"/>
+      <c r="B115" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C115" s="5"/>
+      <c r="D115" s="5"/>
+      <c r="E115" s="5"/>
+      <c r="F115" s="5"/>
+      <c r="G115" s="5"/>
+      <c r="H115" s="5"/>
+      <c r="I115" s="5"/>
+      <c r="J115" s="5"/>
+      <c r="K115" s="5"/>
+      <c r="L115" s="5"/>
+      <c r="M115" s="5"/>
+      <c r="N115" s="5"/>
+      <c r="O115" s="5"/>
+      <c r="P115" s="5"/>
+      <c r="Q115" s="5"/>
+      <c r="R115" s="5"/>
     </row>
     <row r="116" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C116" s="11"/>
-      <c r="D116" s="11"/>
-      <c r="E116" s="11"/>
-      <c r="F116" s="11"/>
-      <c r="G116" s="11"/>
-      <c r="H116" s="11"/>
-      <c r="I116" s="11"/>
-      <c r="J116" s="11"/>
-      <c r="K116" s="11"/>
-      <c r="L116" s="11"/>
-      <c r="M116" s="11"/>
-      <c r="N116" s="11"/>
-      <c r="O116" s="11"/>
-      <c r="P116" s="11"/>
-      <c r="Q116" s="11"/>
-      <c r="R116" s="11"/>
+      <c r="B116" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C116" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D116" s="12"/>
+      <c r="E116" s="12"/>
+      <c r="F116" s="12"/>
+      <c r="G116" s="12"/>
+      <c r="H116" s="12"/>
+      <c r="I116" s="12"/>
+      <c r="J116" s="12"/>
+      <c r="K116" s="12"/>
+      <c r="L116" s="12"/>
+      <c r="M116" s="12"/>
+      <c r="N116" s="12"/>
+      <c r="O116" s="12"/>
+      <c r="P116" s="12"/>
+      <c r="Q116" s="12"/>
+      <c r="R116" s="12"/>
     </row>
     <row r="117" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C117" s="11"/>
-      <c r="D117" s="11"/>
-      <c r="E117" s="11"/>
-      <c r="F117" s="11"/>
-      <c r="G117" s="11"/>
-      <c r="H117" s="11"/>
-      <c r="I117" s="11"/>
-      <c r="J117" s="11"/>
-      <c r="K117" s="11"/>
-      <c r="L117" s="11"/>
-      <c r="M117" s="11"/>
-      <c r="N117" s="11"/>
-      <c r="O117" s="11"/>
-      <c r="P117" s="11"/>
-      <c r="Q117" s="11"/>
-      <c r="R117" s="11"/>
+      <c r="B117" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C117" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D117" s="12"/>
+      <c r="E117" s="12"/>
+      <c r="F117" s="12"/>
+      <c r="G117" s="12"/>
+      <c r="H117" s="12"/>
+      <c r="I117" s="12"/>
+      <c r="J117" s="12"/>
+      <c r="K117" s="12"/>
+      <c r="L117" s="12"/>
+      <c r="M117" s="12"/>
+      <c r="N117" s="12"/>
+      <c r="O117" s="12"/>
+      <c r="P117" s="12"/>
+      <c r="Q117" s="12"/>
+      <c r="R117" s="12"/>
     </row>
     <row r="118" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C118" s="11"/>
-      <c r="D118" s="11"/>
-      <c r="E118" s="11"/>
-      <c r="F118" s="11"/>
-      <c r="G118" s="11"/>
-      <c r="H118" s="11"/>
-      <c r="I118" s="11"/>
-      <c r="J118" s="11"/>
-      <c r="K118" s="11"/>
-      <c r="L118" s="11"/>
-      <c r="M118" s="11"/>
-      <c r="N118" s="11"/>
-      <c r="O118" s="11"/>
-      <c r="P118" s="11"/>
-      <c r="Q118" s="11"/>
-      <c r="R118" s="11"/>
+      <c r="B118" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C118" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D118" s="12"/>
+      <c r="E118" s="12"/>
+      <c r="F118" s="12"/>
+      <c r="G118" s="12"/>
+      <c r="H118" s="12"/>
+      <c r="I118" s="12"/>
+      <c r="J118" s="12"/>
+      <c r="K118" s="12"/>
+      <c r="L118" s="12"/>
+      <c r="M118" s="12"/>
+      <c r="N118" s="12"/>
+      <c r="O118" s="12"/>
+      <c r="P118" s="12"/>
+      <c r="Q118" s="12"/>
+      <c r="R118" s="12"/>
+    </row>
+    <row r="119" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B119" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C119" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D119" s="12"/>
+      <c r="E119" s="12"/>
+      <c r="F119" s="12"/>
+      <c r="G119" s="12"/>
+      <c r="H119" s="12"/>
+      <c r="I119" s="12"/>
+      <c r="J119" s="12"/>
+      <c r="K119" s="12"/>
+      <c r="L119" s="12"/>
+      <c r="M119" s="12"/>
+      <c r="N119" s="12"/>
+      <c r="O119" s="12"/>
+      <c r="P119" s="12"/>
+      <c r="Q119" s="12"/>
+      <c r="R119" s="12"/>
     </row>
     <row r="120" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B120" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C120" s="5"/>
-      <c r="D120" s="5"/>
-      <c r="E120" s="5"/>
-      <c r="F120" s="5"/>
-      <c r="G120" s="5"/>
-      <c r="H120" s="5"/>
-      <c r="I120" s="5"/>
-      <c r="J120" s="5"/>
-      <c r="K120" s="5"/>
-      <c r="L120" s="5"/>
-      <c r="M120" s="5"/>
-      <c r="N120" s="5"/>
-      <c r="O120" s="5"/>
-      <c r="P120" s="5"/>
-      <c r="Q120" s="5"/>
-      <c r="R120" s="5"/>
-      <c r="S120" s="1" t="s">
-        <v>40</v>
-      </c>
+      <c r="B120" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C120" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D120" s="12"/>
+      <c r="E120" s="12"/>
+      <c r="F120" s="12"/>
+      <c r="G120" s="12"/>
+      <c r="H120" s="12"/>
+      <c r="I120" s="12"/>
+      <c r="J120" s="12"/>
+      <c r="K120" s="12"/>
+      <c r="L120" s="12"/>
+      <c r="M120" s="12"/>
+      <c r="N120" s="12"/>
+      <c r="O120" s="12"/>
+      <c r="P120" s="12"/>
+      <c r="Q120" s="12"/>
+      <c r="R120" s="12"/>
     </row>
     <row r="121" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B121" s="6"/>
-      <c r="C121" s="7" t="n">
+      <c r="B121" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C121" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D121" s="12"/>
+      <c r="E121" s="12"/>
+      <c r="F121" s="12"/>
+      <c r="G121" s="12"/>
+      <c r="H121" s="12"/>
+      <c r="I121" s="12"/>
+      <c r="J121" s="12"/>
+      <c r="K121" s="12"/>
+      <c r="L121" s="12"/>
+      <c r="M121" s="12"/>
+      <c r="N121" s="12"/>
+      <c r="O121" s="12"/>
+      <c r="P121" s="12"/>
+      <c r="Q121" s="12"/>
+      <c r="R121" s="12"/>
+    </row>
+    <row r="123" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B123" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C123" s="5"/>
+      <c r="D123" s="5"/>
+      <c r="E123" s="5"/>
+      <c r="F123" s="5"/>
+      <c r="G123" s="5"/>
+      <c r="H123" s="5"/>
+      <c r="I123" s="5"/>
+      <c r="J123" s="5"/>
+      <c r="K123" s="5"/>
+      <c r="L123" s="5"/>
+      <c r="M123" s="5"/>
+      <c r="N123" s="5"/>
+      <c r="O123" s="5"/>
+      <c r="P123" s="5"/>
+      <c r="Q123" s="5"/>
+      <c r="R123" s="5"/>
+    </row>
+    <row r="124" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B124" s="6"/>
+      <c r="C124" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D121" s="7" t="n">
+      <c r="D124" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E121" s="7" t="n">
+      <c r="E124" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F121" s="7" t="n">
+      <c r="F124" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G121" s="7" t="n">
+      <c r="G124" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="H121" s="7" t="n">
+      <c r="H124" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="I121" s="7" t="n">
+      <c r="I124" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="J121" s="7" t="n">
+      <c r="J124" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="K121" s="7" t="n">
+      <c r="K124" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="L121" s="7" t="n">
+      <c r="L124" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="M121" s="7" t="s">
+      <c r="M124" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="N121" s="7" t="s">
+      <c r="N124" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="O121" s="7" t="s">
+      <c r="O124" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="P121" s="7" t="s">
+      <c r="P124" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="Q121" s="7" t="s">
+      <c r="Q124" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="R121" s="7" t="s">
+      <c r="R124" s="7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="122" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B122" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C122" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D122" s="12"/>
-      <c r="E122" s="12"/>
-      <c r="F122" s="12"/>
-      <c r="G122" s="12"/>
-      <c r="H122" s="12"/>
-      <c r="I122" s="12"/>
-      <c r="J122" s="12"/>
-      <c r="K122" s="12"/>
-      <c r="L122" s="12"/>
-      <c r="M122" s="12"/>
-      <c r="N122" s="12"/>
-      <c r="O122" s="12"/>
-      <c r="P122" s="12"/>
-      <c r="Q122" s="12"/>
-      <c r="R122" s="12"/>
-      <c r="S122" s="13" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="123" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B123" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C123" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D123" s="12"/>
-      <c r="E123" s="12"/>
-      <c r="F123" s="12"/>
-      <c r="G123" s="12"/>
-      <c r="H123" s="12"/>
-      <c r="I123" s="12"/>
-      <c r="J123" s="12"/>
-      <c r="K123" s="12"/>
-      <c r="L123" s="12"/>
-      <c r="M123" s="12"/>
-      <c r="N123" s="12"/>
-      <c r="O123" s="12"/>
-      <c r="P123" s="12"/>
-      <c r="Q123" s="12"/>
-      <c r="R123" s="12"/>
-    </row>
-    <row r="124" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B124" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C124" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="D124" s="12"/>
-      <c r="E124" s="12"/>
-      <c r="F124" s="12"/>
-      <c r="G124" s="12"/>
-      <c r="H124" s="12"/>
-      <c r="I124" s="12"/>
-      <c r="J124" s="12"/>
-      <c r="K124" s="12"/>
-      <c r="L124" s="12"/>
-      <c r="M124" s="12"/>
-      <c r="N124" s="12"/>
-      <c r="O124" s="12"/>
-      <c r="P124" s="12"/>
-      <c r="Q124" s="12"/>
-      <c r="R124" s="12"/>
     </row>
     <row r="125" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B125" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C125" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="D125" s="12"/>
-      <c r="E125" s="12"/>
-      <c r="F125" s="12"/>
-      <c r="G125" s="12"/>
-      <c r="H125" s="12"/>
-      <c r="I125" s="12"/>
-      <c r="J125" s="12"/>
-      <c r="K125" s="12"/>
-      <c r="L125" s="12"/>
-      <c r="M125" s="12"/>
-      <c r="N125" s="12"/>
-      <c r="O125" s="12"/>
-      <c r="P125" s="12"/>
-      <c r="Q125" s="12"/>
-      <c r="R125" s="12"/>
+        <v>64</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D125" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E125" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F125" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="S125" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="T125" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="U125" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="V125" s="1" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B126" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C126" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="D126" s="12"/>
-      <c r="E126" s="12"/>
-      <c r="F126" s="12"/>
-      <c r="G126" s="12"/>
-      <c r="H126" s="12"/>
-      <c r="I126" s="12"/>
-      <c r="J126" s="12"/>
-      <c r="K126" s="12"/>
-      <c r="L126" s="12"/>
-      <c r="M126" s="12"/>
-      <c r="N126" s="12"/>
-      <c r="O126" s="12"/>
-      <c r="P126" s="12"/>
-      <c r="Q126" s="12"/>
-      <c r="R126" s="12"/>
+        <v>72</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="S126" s="1" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B127" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C127" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D127" s="12"/>
-      <c r="E127" s="12"/>
-      <c r="F127" s="12"/>
-      <c r="G127" s="12"/>
-      <c r="H127" s="12"/>
-      <c r="I127" s="12"/>
-      <c r="J127" s="12"/>
-      <c r="K127" s="12"/>
-      <c r="L127" s="12"/>
-      <c r="M127" s="12"/>
-      <c r="N127" s="12"/>
-      <c r="O127" s="12"/>
-      <c r="P127" s="12"/>
-      <c r="Q127" s="12"/>
-      <c r="R127" s="12"/>
-    </row>
-    <row r="129" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B129" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C129" s="5"/>
-      <c r="D129" s="5"/>
-      <c r="E129" s="5"/>
-      <c r="F129" s="5"/>
-      <c r="G129" s="5"/>
-      <c r="H129" s="5"/>
-      <c r="I129" s="5"/>
-      <c r="J129" s="5"/>
-      <c r="K129" s="5"/>
-      <c r="L129" s="5"/>
-      <c r="M129" s="5"/>
-      <c r="N129" s="5"/>
-      <c r="O129" s="5"/>
-      <c r="P129" s="5"/>
-      <c r="Q129" s="5"/>
-      <c r="R129" s="5"/>
+        <v>75</v>
+      </c>
+      <c r="C127" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="D127" s="10"/>
+      <c r="E127" s="10"/>
+      <c r="F127" s="10"/>
+      <c r="G127" s="10"/>
+      <c r="H127" s="10"/>
+      <c r="I127" s="10"/>
+      <c r="J127" s="10"/>
+      <c r="K127" s="10"/>
+      <c r="L127" s="10"/>
+      <c r="M127" s="10"/>
+      <c r="N127" s="10"/>
+      <c r="O127" s="10"/>
+      <c r="P127" s="10"/>
+      <c r="Q127" s="10"/>
+      <c r="R127" s="10"/>
+    </row>
+    <row r="128" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B128" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C128" s="10"/>
+      <c r="D128" s="10"/>
+      <c r="E128" s="10"/>
+      <c r="F128" s="10"/>
+      <c r="G128" s="10"/>
+      <c r="H128" s="10"/>
+      <c r="I128" s="10"/>
+      <c r="J128" s="10"/>
+      <c r="K128" s="10"/>
+      <c r="L128" s="10"/>
+      <c r="M128" s="10"/>
+      <c r="N128" s="10"/>
+      <c r="O128" s="10"/>
+      <c r="P128" s="10"/>
+      <c r="Q128" s="10"/>
+      <c r="R128" s="10"/>
     </row>
     <row r="130" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B130" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C130" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D130" s="12"/>
-      <c r="E130" s="12"/>
-      <c r="F130" s="12"/>
-      <c r="G130" s="12"/>
-      <c r="H130" s="12"/>
-      <c r="I130" s="12"/>
-      <c r="J130" s="12"/>
-      <c r="K130" s="12"/>
-      <c r="L130" s="12"/>
-      <c r="M130" s="12"/>
-      <c r="N130" s="12"/>
-      <c r="O130" s="12"/>
-      <c r="P130" s="12"/>
-      <c r="Q130" s="12"/>
-      <c r="R130" s="12"/>
+      <c r="B130" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C130" s="5"/>
+      <c r="D130" s="5"/>
+      <c r="E130" s="5"/>
+      <c r="F130" s="5"/>
+      <c r="G130" s="5"/>
+      <c r="H130" s="5"/>
+      <c r="I130" s="5"/>
+      <c r="J130" s="5"/>
+      <c r="K130" s="5"/>
+      <c r="L130" s="5"/>
+      <c r="M130" s="5"/>
+      <c r="N130" s="5"/>
+      <c r="O130" s="5"/>
+      <c r="P130" s="5"/>
+      <c r="Q130" s="5"/>
+      <c r="R130" s="5"/>
+      <c r="S130" s="1" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="131" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B131" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C131" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D131" s="12"/>
-      <c r="E131" s="12"/>
-      <c r="F131" s="12"/>
-      <c r="G131" s="12"/>
-      <c r="H131" s="12"/>
-      <c r="I131" s="12"/>
-      <c r="J131" s="12"/>
-      <c r="K131" s="12"/>
-      <c r="L131" s="12"/>
-      <c r="M131" s="12"/>
-      <c r="N131" s="12"/>
-      <c r="O131" s="12"/>
-      <c r="P131" s="12"/>
-      <c r="Q131" s="12"/>
-      <c r="R131" s="12"/>
+      <c r="B131" s="6"/>
+      <c r="C131" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D131" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E131" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F131" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G131" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H131" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I131" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J131" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K131" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L131" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M131" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="N131" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O131" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P131" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q131" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R131" s="7" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B132" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C132" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D132" s="12"/>
-      <c r="E132" s="12"/>
-      <c r="F132" s="12"/>
-      <c r="G132" s="12"/>
-      <c r="H132" s="12"/>
-      <c r="I132" s="12"/>
-      <c r="J132" s="12"/>
-      <c r="K132" s="12"/>
-      <c r="L132" s="12"/>
-      <c r="M132" s="12"/>
-      <c r="N132" s="12"/>
-      <c r="O132" s="12"/>
-      <c r="P132" s="12"/>
-      <c r="Q132" s="12"/>
-      <c r="R132" s="12"/>
+        <v>80</v>
+      </c>
+      <c r="C132" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E132" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F132" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G132" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H132" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I132" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J132" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="K132" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L132" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="M132" s="14"/>
+      <c r="N132" s="14"/>
+      <c r="O132" s="14"/>
+      <c r="P132" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q132" s="14"/>
+      <c r="R132" s="14"/>
     </row>
     <row r="133" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B133" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C133" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="D133" s="12"/>
-      <c r="E133" s="12"/>
-      <c r="F133" s="12"/>
-      <c r="G133" s="12"/>
-      <c r="H133" s="12"/>
-      <c r="I133" s="12"/>
-      <c r="J133" s="12"/>
-      <c r="K133" s="12"/>
-      <c r="L133" s="12"/>
-      <c r="M133" s="12"/>
-      <c r="N133" s="12"/>
-      <c r="O133" s="12"/>
-      <c r="P133" s="12"/>
-      <c r="Q133" s="12"/>
-      <c r="R133" s="12"/>
+        <v>82</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E133" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G133" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H133" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I133" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J133" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="K133" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="L133" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="M133" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="N133" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O133" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="P133" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q133" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="R133" s="3" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B134" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C134" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="D134" s="12"/>
-      <c r="E134" s="12"/>
-      <c r="F134" s="12"/>
-      <c r="G134" s="12"/>
-      <c r="H134" s="12"/>
-      <c r="I134" s="12"/>
-      <c r="J134" s="12"/>
-      <c r="K134" s="12"/>
-      <c r="L134" s="12"/>
-      <c r="M134" s="12"/>
-      <c r="N134" s="12"/>
-      <c r="O134" s="12"/>
-      <c r="P134" s="12"/>
-      <c r="Q134" s="12"/>
-      <c r="R134" s="12"/>
-    </row>
-    <row r="135" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B135" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C135" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="D135" s="12"/>
-      <c r="E135" s="12"/>
-      <c r="F135" s="12"/>
-      <c r="G135" s="12"/>
-      <c r="H135" s="12"/>
-      <c r="I135" s="12"/>
-      <c r="J135" s="12"/>
-      <c r="K135" s="12"/>
-      <c r="L135" s="12"/>
-      <c r="M135" s="12"/>
-      <c r="N135" s="12"/>
-      <c r="O135" s="12"/>
-      <c r="P135" s="12"/>
-      <c r="Q135" s="12"/>
-      <c r="R135" s="12"/>
+        <v>93</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E134" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F134" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="G134" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="H134" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I134" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="J134" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="K134" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="L134" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M134" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="N134" s="14"/>
+      <c r="O134" s="14"/>
+      <c r="P134" s="14"/>
+      <c r="Q134" s="14"/>
+      <c r="R134" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B136" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C136" s="5"/>
+      <c r="D136" s="5"/>
+      <c r="E136" s="5"/>
+      <c r="F136" s="5"/>
+      <c r="G136" s="5"/>
+      <c r="H136" s="5"/>
+      <c r="I136" s="5"/>
+      <c r="J136" s="5"/>
+      <c r="K136" s="5"/>
+      <c r="L136" s="5"/>
+      <c r="M136" s="5"/>
+      <c r="N136" s="5"/>
+      <c r="O136" s="5"/>
+      <c r="P136" s="5"/>
+      <c r="Q136" s="5"/>
+      <c r="R136" s="5"/>
     </row>
     <row r="137" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B137" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C137" s="5"/>
-      <c r="D137" s="5"/>
-      <c r="E137" s="5"/>
-      <c r="F137" s="5"/>
-      <c r="G137" s="5"/>
-      <c r="H137" s="5"/>
-      <c r="I137" s="5"/>
-      <c r="J137" s="5"/>
-      <c r="K137" s="5"/>
-      <c r="L137" s="5"/>
-      <c r="M137" s="5"/>
-      <c r="N137" s="5"/>
-      <c r="O137" s="5"/>
-      <c r="P137" s="5"/>
-      <c r="Q137" s="5"/>
-      <c r="R137" s="5"/>
+      <c r="B137" s="6"/>
+      <c r="C137" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D137" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E137" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F137" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G137" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H137" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I137" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J137" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K137" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L137" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M137" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="N137" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O137" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P137" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q137" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R137" s="7" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B138" s="6"/>
-      <c r="C138" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D138" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E138" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F138" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G138" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H138" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I138" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J138" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K138" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L138" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="M138" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="N138" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O138" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P138" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q138" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="R138" s="7" t="s">
-        <v>7</v>
+      <c r="B138" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D138" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E138" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F138" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="S138" s="1" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B139" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C139" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D139" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E139" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="F139" s="3" t="s">
-        <v>71</v>
+        <v>113</v>
+      </c>
+      <c r="R139" s="3" t="s">
+        <v>114</v>
       </c>
       <c r="S139" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="T139" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="U139" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="V139" s="0" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="140" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B140" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C140" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="S140" s="1" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B141" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C141" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="D141" s="10"/>
-      <c r="E141" s="10"/>
-      <c r="F141" s="10"/>
-      <c r="G141" s="10"/>
-      <c r="H141" s="10"/>
-      <c r="I141" s="10"/>
-      <c r="J141" s="10"/>
-      <c r="K141" s="10"/>
-      <c r="L141" s="10"/>
-      <c r="M141" s="10"/>
-      <c r="N141" s="10"/>
-      <c r="O141" s="10"/>
-      <c r="P141" s="10"/>
-      <c r="Q141" s="10"/>
-      <c r="R141" s="10"/>
+      <c r="B141" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C141" s="5"/>
+      <c r="D141" s="5"/>
+      <c r="E141" s="5"/>
+      <c r="F141" s="5"/>
+      <c r="G141" s="5"/>
+      <c r="H141" s="5"/>
+      <c r="I141" s="5"/>
+      <c r="J141" s="5"/>
+      <c r="K141" s="5"/>
+      <c r="L141" s="5"/>
+      <c r="M141" s="5"/>
+      <c r="N141" s="5"/>
+      <c r="O141" s="5"/>
+      <c r="P141" s="5"/>
+      <c r="Q141" s="5"/>
+      <c r="R141" s="5"/>
     </row>
     <row r="142" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B142" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C142" s="10"/>
-      <c r="D142" s="10"/>
-      <c r="E142" s="10"/>
-      <c r="F142" s="10"/>
-      <c r="G142" s="10"/>
-      <c r="H142" s="10"/>
-      <c r="I142" s="10"/>
-      <c r="J142" s="10"/>
-      <c r="K142" s="10"/>
-      <c r="L142" s="10"/>
-      <c r="M142" s="10"/>
-      <c r="N142" s="10"/>
-      <c r="O142" s="10"/>
-      <c r="P142" s="10"/>
-      <c r="Q142" s="10"/>
-      <c r="R142" s="10"/>
-    </row>
-    <row r="144" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B144" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C144" s="5"/>
-      <c r="D144" s="5"/>
-      <c r="E144" s="5"/>
-      <c r="F144" s="5"/>
-      <c r="G144" s="5"/>
-      <c r="H144" s="5"/>
-      <c r="I144" s="5"/>
-      <c r="J144" s="5"/>
-      <c r="K144" s="5"/>
-      <c r="L144" s="5"/>
-      <c r="M144" s="5"/>
-      <c r="N144" s="5"/>
-      <c r="O144" s="5"/>
-      <c r="P144" s="5"/>
-      <c r="Q144" s="5"/>
-      <c r="R144" s="5"/>
-      <c r="S144" s="1" t="s">
-        <v>83</v>
+      <c r="B142" s="6"/>
+      <c r="C142" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D142" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E142" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F142" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G142" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H142" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I142" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J142" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K142" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L142" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M142" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="N142" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O142" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P142" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q142" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R142" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B143" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C143" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="D143" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E143" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F143" s="3" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B145" s="6"/>
-      <c r="C145" s="7" t="n">
+      <c r="B145" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C145" s="5"/>
+      <c r="D145" s="5"/>
+      <c r="E145" s="5"/>
+      <c r="F145" s="5"/>
+      <c r="G145" s="5"/>
+      <c r="H145" s="5"/>
+      <c r="I145" s="5"/>
+      <c r="J145" s="5"/>
+      <c r="K145" s="5"/>
+      <c r="L145" s="5"/>
+      <c r="M145" s="5"/>
+      <c r="N145" s="5"/>
+      <c r="O145" s="5"/>
+      <c r="P145" s="5"/>
+      <c r="Q145" s="5"/>
+      <c r="R145" s="5"/>
+    </row>
+    <row r="146" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B146" s="6"/>
+      <c r="C146" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D145" s="7" t="n">
+      <c r="D146" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E145" s="7" t="n">
+      <c r="E146" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F145" s="7" t="n">
+      <c r="F146" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G145" s="7" t="n">
+      <c r="G146" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="H145" s="7" t="n">
+      <c r="H146" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="I145" s="7" t="n">
+      <c r="I146" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="J145" s="7" t="n">
+      <c r="J146" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="K145" s="7" t="n">
+      <c r="K146" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="L145" s="7" t="n">
+      <c r="L146" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="M145" s="7" t="s">
+      <c r="M146" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="N145" s="7" t="s">
+      <c r="N146" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="O145" s="7" t="s">
+      <c r="O146" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="P145" s="7" t="s">
+      <c r="P146" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="Q145" s="7" t="s">
+      <c r="Q146" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="R145" s="7" t="s">
+      <c r="R146" s="7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="146" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B146" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C146" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D146" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E146" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F146" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G146" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H146" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="I146" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="J146" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="K146" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L146" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="M146" s="14"/>
-      <c r="N146" s="14"/>
-      <c r="O146" s="14"/>
-      <c r="P146" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q146" s="14"/>
-      <c r="R146" s="14"/>
     </row>
     <row r="147" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B147" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C147" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D147" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C147" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E147" s="3" t="s">
+      <c r="E147" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F147" s="3" t="s">
+      <c r="F147" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G147" s="3" t="s">
+      <c r="G147" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="H147" s="3" t="s">
+      <c r="H147" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="I147" s="3" t="s">
+      <c r="I147" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="J147" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="K147" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="L147" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="M147" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="N147" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="O147" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="P147" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q147" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="R147" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="148" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B148" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C148" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="D148" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E148" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="F148" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="G148" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="H148" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="I148" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="J148" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="K148" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L148" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="M148" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="N148" s="14"/>
-      <c r="O148" s="14"/>
-      <c r="P148" s="14"/>
-      <c r="Q148" s="14"/>
-      <c r="R148" s="3" t="s">
-        <v>109</v>
-      </c>
+      <c r="J147" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K147" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L147" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="M147" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="N147" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="O147" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="P147" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q147" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="R147" s="3" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B149" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C149" s="5"/>
+      <c r="D149" s="5"/>
+      <c r="E149" s="5"/>
+      <c r="F149" s="5"/>
+      <c r="G149" s="5"/>
+      <c r="H149" s="5"/>
+      <c r="I149" s="5"/>
+      <c r="J149" s="5"/>
+      <c r="K149" s="5"/>
+      <c r="L149" s="5"/>
+      <c r="M149" s="5"/>
+      <c r="N149" s="5"/>
+      <c r="O149" s="5"/>
+      <c r="P149" s="5"/>
+      <c r="Q149" s="5"/>
+      <c r="R149" s="5"/>
     </row>
     <row r="150" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B150" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C150" s="5"/>
-      <c r="D150" s="5"/>
-      <c r="E150" s="5"/>
-      <c r="F150" s="5"/>
-      <c r="G150" s="5"/>
-      <c r="H150" s="5"/>
-      <c r="I150" s="5"/>
-      <c r="J150" s="5"/>
-      <c r="K150" s="5"/>
-      <c r="L150" s="5"/>
-      <c r="M150" s="5"/>
-      <c r="N150" s="5"/>
-      <c r="O150" s="5"/>
-      <c r="P150" s="5"/>
-      <c r="Q150" s="5"/>
-      <c r="R150" s="5"/>
+      <c r="B150" s="6"/>
+      <c r="C150" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D150" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E150" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F150" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G150" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H150" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I150" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J150" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K150" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="L150" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M150" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="N150" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="O150" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="P150" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q150" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="R150" s="7" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="151" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B151" s="6"/>
-      <c r="C151" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D151" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E151" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F151" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G151" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H151" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I151" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J151" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K151" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L151" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="M151" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="N151" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O151" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P151" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q151" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="R151" s="7" t="s">
-        <v>7</v>
+      <c r="B151" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C151" s="15" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D151" s="3" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E151" s="3" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F151" s="3" t="n">
+        <v>-4</v>
+      </c>
+      <c r="G151" s="3" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H151" s="3" t="n">
+        <v>-6</v>
+      </c>
+      <c r="I151" s="3" t="n">
+        <v>-7</v>
+      </c>
+      <c r="J151" s="3" t="n">
+        <v>-8</v>
+      </c>
+      <c r="K151" s="3" t="n">
+        <v>-9</v>
+      </c>
+      <c r="L151" s="3" t="n">
+        <v>-10</v>
+      </c>
+      <c r="M151" s="3" t="n">
+        <v>-11</v>
+      </c>
+      <c r="N151" s="3" t="n">
+        <v>-12</v>
+      </c>
+      <c r="O151" s="3" t="n">
+        <v>-13</v>
+      </c>
+      <c r="P151" s="3" t="n">
+        <v>-14</v>
+      </c>
+      <c r="Q151" s="3" t="n">
+        <v>-15</v>
+      </c>
+      <c r="R151" s="3" t="n">
+        <v>-16</v>
+      </c>
+      <c r="S151" s="1" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B152" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C152" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="D152" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E152" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="F152" s="3" t="s">
-        <v>115</v>
+        <v>127</v>
+      </c>
+      <c r="C152" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E152" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F152" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G152" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H152" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I152" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="J152" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K152" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="L152" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="M152" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="N152" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="O152" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="P152" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q152" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="R152" s="3" t="n">
+        <v>16</v>
       </c>
       <c r="S152" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="153" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B153" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="R153" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="S153" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="155" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B155" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="C155" s="5"/>
-      <c r="D155" s="5"/>
-      <c r="E155" s="5"/>
-      <c r="F155" s="5"/>
-      <c r="G155" s="5"/>
-      <c r="H155" s="5"/>
-      <c r="I155" s="5"/>
-      <c r="J155" s="5"/>
-      <c r="K155" s="5"/>
-      <c r="L155" s="5"/>
-      <c r="M155" s="5"/>
-      <c r="N155" s="5"/>
-      <c r="O155" s="5"/>
-      <c r="P155" s="5"/>
-      <c r="Q155" s="5"/>
-      <c r="R155" s="5"/>
-    </row>
-    <row r="156" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B156" s="6"/>
-      <c r="C156" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D156" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E156" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F156" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G156" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H156" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I156" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J156" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K156" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L156" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="M156" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="N156" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O156" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P156" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q156" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="R156" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="157" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B157" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C157" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="D157" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="E157" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="F157" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="159" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B159" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C159" s="5"/>
-      <c r="D159" s="5"/>
-      <c r="E159" s="5"/>
-      <c r="F159" s="5"/>
-      <c r="G159" s="5"/>
-      <c r="H159" s="5"/>
-      <c r="I159" s="5"/>
-      <c r="J159" s="5"/>
-      <c r="K159" s="5"/>
-      <c r="L159" s="5"/>
-      <c r="M159" s="5"/>
-      <c r="N159" s="5"/>
-      <c r="O159" s="5"/>
-      <c r="P159" s="5"/>
-      <c r="Q159" s="5"/>
-      <c r="R159" s="5"/>
-    </row>
-    <row r="160" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B160" s="6"/>
-      <c r="C160" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D160" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E160" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F160" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G160" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H160" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I160" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J160" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K160" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L160" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="M160" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="N160" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O160" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P160" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q160" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="R160" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="161" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B161" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="C161" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D161" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E161" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F161" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G161" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H161" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="I161" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="J161" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="K161" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="L161" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="M161" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="N161" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="O161" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="P161" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q161" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="R161" s="3" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="163" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B163" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C163" s="5"/>
-      <c r="D163" s="5"/>
-      <c r="E163" s="5"/>
-      <c r="F163" s="5"/>
-      <c r="G163" s="5"/>
-      <c r="H163" s="5"/>
-      <c r="I163" s="5"/>
-      <c r="J163" s="5"/>
-      <c r="K163" s="5"/>
-      <c r="L163" s="5"/>
-      <c r="M163" s="5"/>
-      <c r="N163" s="5"/>
-      <c r="O163" s="5"/>
-      <c r="P163" s="5"/>
-      <c r="Q163" s="5"/>
-      <c r="R163" s="5"/>
-    </row>
-    <row r="164" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B164" s="6"/>
-      <c r="C164" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D164" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E164" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F164" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G164" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H164" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="I164" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="J164" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="K164" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="L164" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="M164" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="N164" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="O164" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="P164" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q164" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="R164" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="165" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B165" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C165" s="15" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D165" s="3" t="n">
-        <v>-2</v>
-      </c>
-      <c r="E165" s="3" t="n">
-        <v>-3</v>
-      </c>
-      <c r="F165" s="3" t="n">
-        <v>-4</v>
-      </c>
-      <c r="G165" s="3" t="n">
-        <v>-5</v>
-      </c>
-      <c r="H165" s="3" t="n">
-        <v>-6</v>
-      </c>
-      <c r="I165" s="3" t="n">
-        <v>-7</v>
-      </c>
-      <c r="J165" s="3" t="n">
-        <v>-8</v>
-      </c>
-      <c r="K165" s="3" t="n">
-        <v>-9</v>
-      </c>
-      <c r="L165" s="3" t="n">
-        <v>-10</v>
-      </c>
-      <c r="M165" s="3" t="n">
-        <v>-11</v>
-      </c>
-      <c r="N165" s="3" t="n">
-        <v>-12</v>
-      </c>
-      <c r="O165" s="3" t="n">
-        <v>-13</v>
-      </c>
-      <c r="P165" s="3" t="n">
-        <v>-14</v>
-      </c>
-      <c r="Q165" s="3" t="n">
-        <v>-15</v>
-      </c>
-      <c r="R165" s="3" t="n">
-        <v>-16</v>
-      </c>
-      <c r="S165" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="166" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B166" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C166" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D166" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E166" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F166" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G166" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H166" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="I166" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="J166" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="K166" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="L166" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="M166" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="N166" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="O166" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="P166" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q166" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="R166" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="S166" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
+    </row>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="29">
     <mergeCell ref="A1:R1"/>
     <mergeCell ref="B3:R3"/>
     <mergeCell ref="C5:R10"/>
@@ -4956,28 +4693,27 @@
     <mergeCell ref="C21:R84"/>
     <mergeCell ref="C85:R86"/>
     <mergeCell ref="C87:R92"/>
-    <mergeCell ref="C101:R105"/>
-    <mergeCell ref="B120:R120"/>
-    <mergeCell ref="C122:R122"/>
-    <mergeCell ref="C123:R123"/>
-    <mergeCell ref="C124:R124"/>
-    <mergeCell ref="C125:R125"/>
-    <mergeCell ref="C126:R126"/>
-    <mergeCell ref="C127:R127"/>
-    <mergeCell ref="B129:R129"/>
-    <mergeCell ref="C130:R130"/>
-    <mergeCell ref="C131:R131"/>
-    <mergeCell ref="C132:R132"/>
-    <mergeCell ref="C133:R133"/>
-    <mergeCell ref="C134:R134"/>
-    <mergeCell ref="C135:R135"/>
-    <mergeCell ref="B137:R137"/>
-    <mergeCell ref="C141:R142"/>
-    <mergeCell ref="B144:R144"/>
-    <mergeCell ref="B150:R150"/>
-    <mergeCell ref="B155:R155"/>
-    <mergeCell ref="B159:R159"/>
-    <mergeCell ref="B163:R163"/>
+    <mergeCell ref="B106:R106"/>
+    <mergeCell ref="C108:R108"/>
+    <mergeCell ref="C109:R109"/>
+    <mergeCell ref="C110:R110"/>
+    <mergeCell ref="C111:R111"/>
+    <mergeCell ref="C112:R112"/>
+    <mergeCell ref="C113:R113"/>
+    <mergeCell ref="B115:R115"/>
+    <mergeCell ref="C116:R116"/>
+    <mergeCell ref="C117:R117"/>
+    <mergeCell ref="C118:R118"/>
+    <mergeCell ref="C119:R119"/>
+    <mergeCell ref="C120:R120"/>
+    <mergeCell ref="C121:R121"/>
+    <mergeCell ref="B123:R123"/>
+    <mergeCell ref="C127:R128"/>
+    <mergeCell ref="B130:R130"/>
+    <mergeCell ref="B136:R136"/>
+    <mergeCell ref="B141:R141"/>
+    <mergeCell ref="B145:R145"/>
+    <mergeCell ref="B149:R149"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4994,7 +4730,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R37"/>
+  <dimension ref="A1:T37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15.4" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.71"/>
@@ -5004,7 +4740,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -5099,7 +4835,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D6" s="17"/>
       <c r="E6" s="17"/>
@@ -5116,6 +4852,9 @@
       <c r="P6" s="17"/>
       <c r="Q6" s="17"/>
       <c r="R6" s="17"/>
+      <c r="T6" s="0" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="2" t="n">
@@ -5452,10 +5191,10 @@
     </row>
     <row r="23" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
@@ -5475,7 +5214,7 @@
     </row>
     <row r="24" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -5496,7 +5235,7 @@
     </row>
     <row r="25" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -5517,7 +5256,7 @@
     </row>
     <row r="26" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="19" t="s">
-        <v>36</v>
+        <v>136</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
@@ -5538,7 +5277,7 @@
     </row>
     <row r="27" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
@@ -5559,7 +5298,7 @@
     </row>
     <row r="28" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
@@ -5580,7 +5319,7 @@
     </row>
     <row r="29" customFormat="false" ht="15.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>

</xml_diff>